<commit_message>
Drop non-artwork pages and duplicate shots from the folk collection
The folk source document mixed 21 pages that are not works to sell in with
the paintings: a locator map, blank canvas backs, a workshop wall, a scroll
on the floor, detail crops, and ten angled snapshots of paintings that are
also present as flat scans. They are now excluded at the build step, and
build-catalog prunes assets left behind by anything excluded.

Folk goes from 86 to 65 works, the catalogue from 129 to 108, and the
artist card for Folk & Tribal Masters now shows a painting instead of the
map of India.
</commit_message>
<xml_diff>
--- a/Indus Art Collection - Catalogue.xlsx
+++ b/Indus Art Collection - Catalogue.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1040" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="872" uniqueCount="160">
   <si>
     <t>ID (do not edit)</t>
   </si>
@@ -94,7 +94,7 @@
     <t>gopal-naskar-4</t>
   </si>
   <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-7</t>
+    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-10</t>
   </si>
   <si>
     <t>Folk &amp; Tribal Masters</t>
@@ -103,21 +103,6 @@
     <t>Folk</t>
   </si>
   <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-8</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-9</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-10</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-11</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-12</t>
-  </si>
-  <si>
     <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-13</t>
   </si>
   <si>
@@ -139,24 +124,9 @@
     <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-19</t>
   </si>
   <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-20</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-21</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-22</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-23</t>
-  </si>
-  <si>
     <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-24</t>
   </si>
   <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-25</t>
-  </si>
-  <si>
     <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-26</t>
   </si>
   <si>
@@ -178,18 +148,9 @@
     <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-33</t>
   </si>
   <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-34</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-35</t>
-  </si>
-  <si>
     <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-36</t>
   </si>
   <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-37</t>
-  </si>
-  <si>
     <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-38</t>
   </si>
   <si>
@@ -232,9 +193,6 @@
     <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-51</t>
   </si>
   <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-52</t>
-  </si>
-  <si>
     <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-53</t>
   </si>
   <si>
@@ -244,15 +202,9 @@
     <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-55</t>
   </si>
   <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-56</t>
-  </si>
-  <si>
     <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-57</t>
   </si>
   <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-58</t>
-  </si>
-  <si>
     <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-59</t>
   </si>
   <si>
@@ -265,9 +217,6 @@
     <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-62</t>
   </si>
   <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-63</t>
-  </si>
-  <si>
     <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-64</t>
   </si>
   <si>
@@ -283,15 +232,9 @@
     <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-68</t>
   </si>
   <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-69</t>
-  </si>
-  <si>
     <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-70</t>
   </si>
   <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-71</t>
-  </si>
-  <si>
     <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-72</t>
   </si>
   <si>
@@ -322,13 +265,7 @@
     <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-81</t>
   </si>
   <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-82</t>
-  </si>
-  <si>
     <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-83</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-84</t>
   </si>
   <si>
     <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-85</t>
@@ -959,7 +896,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H130"/>
+  <dimension ref="A1:H109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
@@ -2927,22 +2864,22 @@
         <v>94</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>28</v>
+        <v>95</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D76" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>14</v>
+        <v>96</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G76" s="2" t="s">
-        <v>14</v>
+        <v>97</v>
       </c>
       <c r="H76" s="4" t="s">
         <v>15</v>
@@ -2950,25 +2887,25 @@
     </row>
     <row r="77" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B77" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B77" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="C77" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D77" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>14</v>
+        <v>96</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G77" s="2" t="s">
-        <v>14</v>
+        <v>97</v>
       </c>
       <c r="H77" s="4" t="s">
         <v>15</v>
@@ -2976,25 +2913,25 @@
     </row>
     <row r="78" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>28</v>
+        <v>95</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D78" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>14</v>
+        <v>100</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G78" s="2" t="s">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="H78" s="4" t="s">
         <v>15</v>
@@ -3002,25 +2939,25 @@
     </row>
     <row r="79" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>28</v>
+        <v>95</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D79" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>14</v>
+        <v>100</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G79" s="2" t="s">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="H79" s="4" t="s">
         <v>15</v>
@@ -3028,13 +2965,13 @@
     </row>
     <row r="80" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>28</v>
+        <v>104</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>29</v>
+        <v>105</v>
       </c>
       <c r="D80" s="2" t="s">
         <v>14</v>
@@ -3054,13 +2991,13 @@
     </row>
     <row r="81" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>28</v>
+        <v>104</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>29</v>
+        <v>105</v>
       </c>
       <c r="D81" s="2" t="s">
         <v>14</v>
@@ -3080,13 +3017,13 @@
     </row>
     <row r="82" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>28</v>
+        <v>104</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>29</v>
+        <v>105</v>
       </c>
       <c r="D82" s="2" t="s">
         <v>14</v>
@@ -3106,13 +3043,13 @@
     </row>
     <row r="83" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>28</v>
+        <v>104</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>29</v>
+        <v>105</v>
       </c>
       <c r="D83" s="2" t="s">
         <v>14</v>
@@ -3132,22 +3069,22 @@
     </row>
     <row r="84" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>28</v>
+        <v>110</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>14</v>
+        <v>111</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>14</v>
+        <v>112</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>14</v>
+        <v>113</v>
       </c>
       <c r="G84" s="2" t="s">
         <v>14</v>
@@ -3158,22 +3095,22 @@
     </row>
     <row r="85" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>28</v>
+        <v>110</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>14</v>
+        <v>115</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>14</v>
+        <v>112</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G85" s="2" t="s">
         <v>14</v>
@@ -3184,22 +3121,22 @@
     </row>
     <row r="86" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>28</v>
+        <v>110</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D86" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>14</v>
+        <v>117</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G86" s="2" t="s">
         <v>14</v>
@@ -3210,22 +3147,22 @@
     </row>
     <row r="87" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>28</v>
+        <v>110</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D87" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>14</v>
+        <v>117</v>
       </c>
       <c r="F87" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G87" s="2" t="s">
         <v>14</v>
@@ -3236,22 +3173,22 @@
     </row>
     <row r="88" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>28</v>
+        <v>110</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D88" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>14</v>
+        <v>117</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G88" s="2" t="s">
         <v>14</v>
@@ -3262,22 +3199,22 @@
     </row>
     <row r="89" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>28</v>
+        <v>110</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D89" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>14</v>
+        <v>117</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G89" s="2" t="s">
         <v>14</v>
@@ -3288,22 +3225,22 @@
     </row>
     <row r="90" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>28</v>
+        <v>110</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D90" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>14</v>
+        <v>117</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G90" s="2" t="s">
         <v>14</v>
@@ -3314,22 +3251,22 @@
     </row>
     <row r="91" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>28</v>
+        <v>110</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D91" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>14</v>
+        <v>117</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G91" s="2" t="s">
         <v>14</v>
@@ -3340,19 +3277,19 @@
     </row>
     <row r="92" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>28</v>
+        <v>124</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>29</v>
+        <v>105</v>
       </c>
       <c r="D92" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>14</v>
+        <v>125</v>
       </c>
       <c r="F92" s="2" t="s">
         <v>14</v>
@@ -3366,19 +3303,19 @@
     </row>
     <row r="93" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>28</v>
+        <v>124</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>29</v>
+        <v>105</v>
       </c>
       <c r="D93" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>14</v>
+        <v>127</v>
       </c>
       <c r="F93" s="2" t="s">
         <v>14</v>
@@ -3392,19 +3329,19 @@
     </row>
     <row r="94" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>28</v>
+        <v>124</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>29</v>
+        <v>105</v>
       </c>
       <c r="D94" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>14</v>
+        <v>129</v>
       </c>
       <c r="F94" s="2" t="s">
         <v>14</v>
@@ -3418,19 +3355,19 @@
     </row>
     <row r="95" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>28</v>
+        <v>124</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>29</v>
+        <v>105</v>
       </c>
       <c r="D95" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>14</v>
+        <v>131</v>
       </c>
       <c r="F95" s="2" t="s">
         <v>14</v>
@@ -3444,19 +3381,19 @@
     </row>
     <row r="96" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>28</v>
+        <v>133</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D96" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>14</v>
+        <v>134</v>
       </c>
       <c r="F96" s="2" t="s">
         <v>14</v>
@@ -3470,10 +3407,10 @@
     </row>
     <row r="97" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
-        <v>115</v>
+        <v>135</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>116</v>
+        <v>133</v>
       </c>
       <c r="C97" s="2" t="s">
         <v>10</v>
@@ -3482,13 +3419,13 @@
         <v>14</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="F97" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>118</v>
+        <v>14</v>
       </c>
       <c r="H97" s="4" t="s">
         <v>15</v>
@@ -3496,10 +3433,10 @@
     </row>
     <row r="98" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>116</v>
+        <v>138</v>
       </c>
       <c r="C98" s="2" t="s">
         <v>10</v>
@@ -3508,13 +3445,13 @@
         <v>14</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>117</v>
+        <v>14</v>
       </c>
       <c r="F98" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>118</v>
+        <v>14</v>
       </c>
       <c r="H98" s="4" t="s">
         <v>15</v>
@@ -3522,10 +3459,10 @@
     </row>
     <row r="99" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
-        <v>120</v>
+        <v>139</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>116</v>
+        <v>138</v>
       </c>
       <c r="C99" s="2" t="s">
         <v>10</v>
@@ -3534,13 +3471,13 @@
         <v>14</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>121</v>
+        <v>14</v>
       </c>
       <c r="F99" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>122</v>
+        <v>14</v>
       </c>
       <c r="H99" s="4" t="s">
         <v>15</v>
@@ -3548,10 +3485,10 @@
     </row>
     <row r="100" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="s">
-        <v>123</v>
+        <v>140</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>116</v>
+        <v>138</v>
       </c>
       <c r="C100" s="2" t="s">
         <v>10</v>
@@ -3560,13 +3497,13 @@
         <v>14</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>121</v>
+        <v>14</v>
       </c>
       <c r="F100" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G100" s="2" t="s">
-        <v>122</v>
+        <v>14</v>
       </c>
       <c r="H100" s="4" t="s">
         <v>15</v>
@@ -3574,13 +3511,13 @@
     </row>
     <row r="101" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="3" t="s">
-        <v>124</v>
+        <v>141</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>126</v>
+        <v>10</v>
       </c>
       <c r="D101" s="2" t="s">
         <v>14</v>
@@ -3600,22 +3537,22 @@
     </row>
     <row r="102" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="3" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>126</v>
+        <v>10</v>
       </c>
       <c r="D102" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>14</v>
+        <v>144</v>
       </c>
       <c r="F102" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G102" s="2" t="s">
         <v>14</v>
@@ -3626,25 +3563,25 @@
     </row>
     <row r="103" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
-        <v>128</v>
+        <v>145</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>126</v>
+        <v>10</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>14</v>
+        <v>146</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>14</v>
+        <v>147</v>
       </c>
       <c r="F103" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G103" s="2" t="s">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="H103" s="4" t="s">
         <v>15</v>
@@ -3652,25 +3589,25 @@
     </row>
     <row r="104" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="3" t="s">
-        <v>129</v>
+        <v>148</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>126</v>
+        <v>10</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>14</v>
+        <v>149</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>14</v>
+        <v>147</v>
       </c>
       <c r="F104" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G104" s="2" t="s">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="H104" s="4" t="s">
         <v>15</v>
@@ -3678,25 +3615,25 @@
     </row>
     <row r="105" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="3" t="s">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="C105" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="F105" s="2" t="s">
-        <v>134</v>
+        <v>13</v>
       </c>
       <c r="G105" s="2" t="s">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="H105" s="4" t="s">
         <v>15</v>
@@ -3704,25 +3641,25 @@
     </row>
     <row r="106" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="3" t="s">
-        <v>135</v>
+        <v>152</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="C106" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>136</v>
+        <v>153</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="F106" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G106" s="2" t="s">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="H106" s="4" t="s">
         <v>15</v>
@@ -3730,25 +3667,25 @@
     </row>
     <row r="107" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="3" t="s">
-        <v>137</v>
+        <v>154</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="C107" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>14</v>
+        <v>155</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="F107" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G107" s="2" t="s">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="H107" s="4" t="s">
         <v>15</v>
@@ -3756,19 +3693,19 @@
     </row>
     <row r="108" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="3" t="s">
-        <v>139</v>
+        <v>156</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="C108" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>14</v>
+        <v>157</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>138</v>
+        <v>158</v>
       </c>
       <c r="F108" s="2" t="s">
         <v>13</v>
@@ -3782,19 +3719,19 @@
     </row>
     <row r="109" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="3" t="s">
-        <v>140</v>
+        <v>159</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="C109" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>14</v>
+        <v>157</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>138</v>
+        <v>158</v>
       </c>
       <c r="F109" s="2" t="s">
         <v>13</v>
@@ -3806,554 +3743,8 @@
         <v>15</v>
       </c>
     </row>
-    <row r="110" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="B110" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C110" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D110" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E110" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="F110" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G110" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H110" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="111" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A111" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="B111" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C111" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D111" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E111" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="F111" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G111" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H111" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="112" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A112" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="B112" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C112" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D112" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E112" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="F112" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G112" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H112" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="113" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A113" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="B113" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="C113" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="D113" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E113" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="F113" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G113" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H113" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="114" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A114" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="B114" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="C114" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="D114" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E114" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="F114" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G114" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H114" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="115" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A115" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="B115" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="C115" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="D115" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E115" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="F115" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G115" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H115" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="116" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A116" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="B116" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="C116" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="D116" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E116" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F116" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G116" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H116" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="117" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A117" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="B117" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="C117" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D117" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E117" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="F117" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G117" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H117" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="118" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="B118" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="C118" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D118" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E118" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="F118" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G118" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H118" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="119" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A119" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="B119" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="C119" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D119" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E119" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F119" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G119" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H119" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="120" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A120" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="B120" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="C120" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D120" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E120" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F120" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G120" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H120" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="121" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A121" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="B121" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="C121" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D121" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E121" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F121" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G121" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H121" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="122" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A122" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="B122" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="C122" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D122" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E122" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F122" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G122" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H122" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="123" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A123" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="B123" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="C123" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D123" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E123" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="F123" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G123" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H123" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="124" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A124" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="B124" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="C124" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D124" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="E124" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="F124" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G124" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="H124" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="125" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A125" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="B125" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="C125" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D125" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="E125" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="F125" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G125" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="H125" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="126" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A126" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="B126" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="C126" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D126" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="E126" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="F126" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G126" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="H126" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="127" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A127" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="B127" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="C127" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D127" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="E127" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="F127" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G127" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="H127" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="128" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A128" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="B128" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="C128" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D128" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="E128" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="F128" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G128" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="H128" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="129" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A129" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="B129" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="C129" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D129" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="E129" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="F129" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G129" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H129" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="130" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A130" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="B130" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="C130" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D130" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="E130" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="F130" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G130" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H130" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H130"/>
+  <autoFilter ref="A1:H109"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Add a single npm run add-art command for publishing artwork
Adding a painting previously meant running the catalogue script, building,
then committing and pushing by hand. This wraps those steps in one command
that reports what it found in plain English, refuses to publish if the site
does not build, and asks before going live.

It also turns the catalogue script's "no artist for X" warning into a stop
with instructions, since an unmatched filename otherwise leaves the painting
silently missing from the site.

The README now documents adding paintings, writing descriptions and adding a
new artist without assuming any development experience.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Uv8R3RW9M9MhGG8c2qV64h
</commit_message>
<xml_diff>
--- a/Indus Art Collection - Catalogue.xlsx
+++ b/Indus Art Collection - Catalogue.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="872" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="141">
   <si>
     <t>ID (do not edit)</t>
   </si>
@@ -340,48 +340,6 @@
     <t>m-salim-painting-4</t>
   </si>
   <si>
-    <t>mehnaaz-bano-painting-1</t>
-  </si>
-  <si>
-    <t>Mainaz Bano</t>
-  </si>
-  <si>
-    <t>Inheritance 1</t>
-  </si>
-  <si>
-    <t>8 x 8 in</t>
-  </si>
-  <si>
-    <t>Mixed media on canvas</t>
-  </si>
-  <si>
-    <t>mehnaaz-bano-painting-2</t>
-  </si>
-  <si>
-    <t>Inheritance 10</t>
-  </si>
-  <si>
-    <t>mehnaaz-bano-painting-3</t>
-  </si>
-  <si>
-    <t>12 x 12 in</t>
-  </si>
-  <si>
-    <t>mehnaaz-bano-painting-4</t>
-  </si>
-  <si>
-    <t>mehnaaz-bano-painting-5</t>
-  </si>
-  <si>
-    <t>mehnaaz-bano-painting-6</t>
-  </si>
-  <si>
-    <t>mehnaaz-bano-painting-7</t>
-  </si>
-  <si>
-    <t>mehnaaz-bano-painting-8</t>
-  </si>
-  <si>
     <t>n-k-mishra-1</t>
   </si>
   <si>
@@ -451,34 +409,19 @@
     <t>umesh-ji-2</t>
   </si>
   <si>
-    <t>Painting 10/2025</t>
-  </si>
-  <si>
     <t>36 x 72 in</t>
   </si>
   <si>
     <t>umesh-ji-3</t>
   </si>
   <si>
-    <t>Painting 11/2025</t>
-  </si>
-  <si>
     <t>umesh-ji-4</t>
   </si>
   <si>
-    <t>Painting 12/2025</t>
-  </si>
-  <si>
     <t>umesh-ji-5</t>
   </si>
   <si>
-    <t>Painting 15/2025</t>
-  </si>
-  <si>
     <t>umesh-ji-6</t>
-  </si>
-  <si>
-    <t>Painting 17/2025</t>
   </si>
   <si>
     <t>umesh-kumar-saxena-painting-1-1</t>
@@ -896,7 +839,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H109"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
@@ -3075,16 +3018,16 @@
         <v>110</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>10</v>
+        <v>105</v>
       </c>
       <c r="D84" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E84" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="E84" s="2" t="s">
-        <v>112</v>
-      </c>
       <c r="F84" s="2" t="s">
-        <v>113</v>
+        <v>14</v>
       </c>
       <c r="G84" s="2" t="s">
         <v>14</v>
@@ -3095,22 +3038,22 @@
     </row>
     <row r="85" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>110</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>10</v>
+        <v>105</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>115</v>
+        <v>14</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G85" s="2" t="s">
         <v>14</v>
@@ -3121,22 +3064,22 @@
     </row>
     <row r="86" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>110</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>10</v>
+        <v>105</v>
       </c>
       <c r="D86" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G86" s="2" t="s">
         <v>14</v>
@@ -3147,13 +3090,13 @@
     </row>
     <row r="87" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B87" s="2" t="s">
         <v>110</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>10</v>
+        <v>105</v>
       </c>
       <c r="D87" s="2" t="s">
         <v>14</v>
@@ -3162,7 +3105,7 @@
         <v>117</v>
       </c>
       <c r="F87" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G87" s="2" t="s">
         <v>14</v>
@@ -3173,10 +3116,10 @@
     </row>
     <row r="88" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B88" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="B88" s="2" t="s">
-        <v>110</v>
       </c>
       <c r="C88" s="2" t="s">
         <v>10</v>
@@ -3185,10 +3128,10 @@
         <v>14</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G88" s="2" t="s">
         <v>14</v>
@@ -3199,10 +3142,10 @@
     </row>
     <row r="89" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="C89" s="2" t="s">
         <v>10</v>
@@ -3211,10 +3154,10 @@
         <v>14</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G89" s="2" t="s">
         <v>14</v>
@@ -3225,10 +3168,10 @@
     </row>
     <row r="90" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="C90" s="2" t="s">
         <v>10</v>
@@ -3237,10 +3180,10 @@
         <v>14</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>117</v>
+        <v>14</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G90" s="2" t="s">
         <v>14</v>
@@ -3251,10 +3194,10 @@
     </row>
     <row r="91" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="C91" s="2" t="s">
         <v>10</v>
@@ -3263,10 +3206,10 @@
         <v>14</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>117</v>
+        <v>14</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G91" s="2" t="s">
         <v>14</v>
@@ -3277,19 +3220,19 @@
     </row>
     <row r="92" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>124</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="D92" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>125</v>
+        <v>14</v>
       </c>
       <c r="F92" s="2" t="s">
         <v>14</v>
@@ -3303,19 +3246,19 @@
     </row>
     <row r="93" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B93" s="2" t="s">
         <v>124</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="D93" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>127</v>
+        <v>14</v>
       </c>
       <c r="F93" s="2" t="s">
         <v>14</v>
@@ -3332,19 +3275,19 @@
         <v>128</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="D94" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F94" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G94" s="2" t="s">
         <v>14</v>
@@ -3355,25 +3298,25 @@
     </row>
     <row r="95" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="D95" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F95" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="H95" s="4" t="s">
         <v>15</v>
@@ -3381,10 +3324,10 @@
     </row>
     <row r="96" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C96" s="2" t="s">
         <v>10</v>
@@ -3393,13 +3336,13 @@
         <v>14</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F96" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G96" s="2" t="s">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="H96" s="4" t="s">
         <v>15</v>
@@ -3407,10 +3350,10 @@
     </row>
     <row r="97" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C97" s="2" t="s">
         <v>10</v>
@@ -3419,13 +3362,13 @@
         <v>14</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="F97" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="H97" s="4" t="s">
         <v>15</v>
@@ -3433,10 +3376,10 @@
     </row>
     <row r="98" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="C98" s="2" t="s">
         <v>10</v>
@@ -3445,13 +3388,13 @@
         <v>14</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>14</v>
+        <v>132</v>
       </c>
       <c r="F98" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="H98" s="4" t="s">
         <v>15</v>
@@ -3459,10 +3402,10 @@
     </row>
     <row r="99" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="C99" s="2" t="s">
         <v>10</v>
@@ -3471,13 +3414,13 @@
         <v>14</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>14</v>
+        <v>132</v>
       </c>
       <c r="F99" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="H99" s="4" t="s">
         <v>15</v>
@@ -3485,22 +3428,22 @@
     </row>
     <row r="100" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="C100" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>14</v>
+        <v>138</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>14</v>
+        <v>139</v>
       </c>
       <c r="F100" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G100" s="2" t="s">
         <v>14</v>
@@ -3511,22 +3454,22 @@
     </row>
     <row r="101" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="C101" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>14</v>
+        <v>138</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>14</v>
+        <v>139</v>
       </c>
       <c r="F101" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G101" s="2" t="s">
         <v>14</v>
@@ -3535,216 +3478,8 @@
         <v>15</v>
       </c>
     </row>
-    <row r="102" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="B102" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C102" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D102" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E102" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="F102" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G102" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H102" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="103" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A103" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="B103" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C103" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D103" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="E103" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="F103" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G103" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="H103" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="104" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="B104" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C104" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D104" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="E104" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="F104" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G104" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="H104" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="105" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="B105" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C105" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D105" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="E105" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="F105" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G105" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="H105" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="106" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A106" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="B106" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C106" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D106" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="E106" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="F106" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G106" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="H106" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="107" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A107" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="B107" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C107" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D107" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="E107" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="F107" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G107" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="H107" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="108" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A108" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="B108" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C108" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D108" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="E108" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="F108" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G108" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H108" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="109" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="B109" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C109" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D109" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="E109" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="F109" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G109" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H109" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H109"/>
+  <autoFilter ref="A1:H101"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Show each painting's details in the zoom view, and stop losing spreadsheet edits
Opening a painting now lists artist, medium, size and price, each labelled,
with anything not yet catalogued offered On request so every work reads the
same way. An Enquire Now button carries the painting into the contact form,
which arrives naming the work in its message and subject line.

The catalogue script also read back only the Description column when it
regenerated the spreadsheet, so Title, Size, Medium and Year typed in by hand
were silently discarded on the next run. It now carries back all five editable
columns, and an empty cell falls back to the caption reading rather than
wiping it. The column headings say which are editable.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Uv8R3RW9M9MhGG8c2qV64h
</commit_message>
<xml_diff>
--- a/Indus Art Collection - Catalogue.xlsx
+++ b/Indus Art Collection - Catalogue.xlsx
@@ -16,25 +16,25 @@
     <t>ID (do not edit)</t>
   </si>
   <si>
-    <t>Artist</t>
-  </si>
-  <si>
-    <t>Style</t>
-  </si>
-  <si>
-    <t>Title</t>
-  </si>
-  <si>
-    <t>Size</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>Description (fill this in)</t>
+    <t>Artist (do not edit)</t>
+  </si>
+  <si>
+    <t>Style (do not edit)</t>
+  </si>
+  <si>
+    <t>Title (editable)</t>
+  </si>
+  <si>
+    <t>Size (editable)</t>
+  </si>
+  <si>
+    <t>Medium (editable)</t>
+  </si>
+  <si>
+    <t>Year (editable)</t>
+  </si>
+  <si>
+    <t>Description (editable)</t>
   </si>
   <si>
     <t>ashok-rathod-painting-1</t>

</xml_diff>

<commit_message>
Update the gallery catalogue
</commit_message>
<xml_diff>
--- a/Indus Art Collection - Catalogue.xlsx
+++ b/Indus Art Collection - Catalogue.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="150">
   <si>
     <t>ID (do not edit)</t>
   </si>
@@ -85,6 +85,9 @@
     <t>Gopal Naskar</t>
   </si>
   <si>
+    <t>Details on request</t>
+  </si>
+  <si>
     <t>gopal-naskar-2</t>
   </si>
   <si>
@@ -301,6 +304,9 @@
     <t>Kandan G</t>
   </si>
   <si>
+    <t>Banaras Series</t>
+  </si>
+  <si>
     <t>24 x 48 in / 61 x 122 cm</t>
   </si>
   <si>
@@ -331,6 +337,12 @@
     <t>Traditional</t>
   </si>
   <si>
+    <t>Landscape</t>
+  </si>
+  <si>
+    <t>Mix Medium</t>
+  </si>
+  <si>
     <t>m-salim-painting-2</t>
   </si>
   <si>
@@ -349,21 +361,33 @@
     <t>21.5 x 15 in</t>
   </si>
   <si>
+    <t>Water colour and gouache on paper</t>
+  </si>
+  <si>
     <t>n-k-mishra-2</t>
   </si>
   <si>
+    <t>Parvati and Ganesha</t>
+  </si>
+  <si>
     <t>13.2 x 7.1 in</t>
   </si>
   <si>
     <t>n-k-mishra-3</t>
   </si>
   <si>
+    <t>Ganesh</t>
+  </si>
+  <si>
     <t>12.5 x 8.5 in</t>
   </si>
   <si>
     <t>n-k-mishra-4</t>
   </si>
   <si>
+    <t>Hanuman</t>
+  </si>
+  <si>
     <t>19.5 x 19.5 in</t>
   </si>
   <si>
@@ -386,6 +410,9 @@
   </si>
   <si>
     <t>Umendra P. Singh</t>
+  </si>
+  <si>
+    <t>Oil on Canvas</t>
   </si>
   <si>
     <t>umendra-p-singh-2</t>
@@ -1019,13 +1046,13 @@
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>14</v>
@@ -1036,7 +1063,7 @@
     </row>
     <row r="8" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>23</v>
@@ -1045,13 +1072,13 @@
         <v>10</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>14</v>
@@ -1062,7 +1089,7 @@
     </row>
     <row r="9" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>23</v>
@@ -1071,13 +1098,13 @@
         <v>10</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>14</v>
@@ -1088,7 +1115,7 @@
     </row>
     <row r="10" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>23</v>
@@ -1097,13 +1124,13 @@
         <v>10</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>14</v>
@@ -1114,22 +1141,22 @@
     </row>
     <row r="11" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>14</v>
@@ -1140,22 +1167,22 @@
     </row>
     <row r="12" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>14</v>
@@ -1166,22 +1193,22 @@
     </row>
     <row r="13" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>14</v>
@@ -1192,22 +1219,22 @@
     </row>
     <row r="14" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>14</v>
@@ -1218,22 +1245,22 @@
     </row>
     <row r="15" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>14</v>
@@ -1244,22 +1271,22 @@
     </row>
     <row r="16" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>14</v>
@@ -1270,22 +1297,22 @@
     </row>
     <row r="17" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>14</v>
@@ -1296,22 +1323,22 @@
     </row>
     <row r="18" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>14</v>
@@ -1322,22 +1349,22 @@
     </row>
     <row r="19" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>14</v>
@@ -1348,22 +1375,22 @@
     </row>
     <row r="20" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>14</v>
@@ -1374,22 +1401,22 @@
     </row>
     <row r="21" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>14</v>
@@ -1400,22 +1427,22 @@
     </row>
     <row r="22" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>14</v>
@@ -1426,22 +1453,22 @@
     </row>
     <row r="23" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>14</v>
@@ -1452,22 +1479,22 @@
     </row>
     <row r="24" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>14</v>
@@ -1478,22 +1505,22 @@
     </row>
     <row r="25" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>14</v>
@@ -1504,22 +1531,22 @@
     </row>
     <row r="26" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>14</v>
@@ -1530,22 +1557,22 @@
     </row>
     <row r="27" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>14</v>
@@ -1556,22 +1583,22 @@
     </row>
     <row r="28" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>14</v>
@@ -1582,22 +1609,22 @@
     </row>
     <row r="29" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>14</v>
@@ -1608,22 +1635,22 @@
     </row>
     <row r="30" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>14</v>
@@ -1634,22 +1661,22 @@
     </row>
     <row r="31" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>14</v>
@@ -1660,22 +1687,22 @@
     </row>
     <row r="32" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>14</v>
@@ -1686,22 +1713,22 @@
     </row>
     <row r="33" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G33" s="2" t="s">
         <v>14</v>
@@ -1712,22 +1739,22 @@
     </row>
     <row r="34" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>14</v>
@@ -1738,22 +1765,22 @@
     </row>
     <row r="35" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>14</v>
@@ -1764,22 +1791,22 @@
     </row>
     <row r="36" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>14</v>
@@ -1790,22 +1817,22 @@
     </row>
     <row r="37" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>14</v>
@@ -1816,22 +1843,22 @@
     </row>
     <row r="38" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G38" s="2" t="s">
         <v>14</v>
@@ -1842,22 +1869,22 @@
     </row>
     <row r="39" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G39" s="2" t="s">
         <v>14</v>
@@ -1868,22 +1895,22 @@
     </row>
     <row r="40" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>14</v>
@@ -1894,22 +1921,22 @@
     </row>
     <row r="41" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G41" s="2" t="s">
         <v>14</v>
@@ -1920,22 +1947,22 @@
     </row>
     <row r="42" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>14</v>
@@ -1946,22 +1973,22 @@
     </row>
     <row r="43" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G43" s="2" t="s">
         <v>14</v>
@@ -1972,22 +1999,22 @@
     </row>
     <row r="44" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G44" s="2" t="s">
         <v>14</v>
@@ -1998,22 +2025,22 @@
     </row>
     <row r="45" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G45" s="2" t="s">
         <v>14</v>
@@ -2024,22 +2051,22 @@
     </row>
     <row r="46" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>14</v>
@@ -2050,22 +2077,22 @@
     </row>
     <row r="47" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G47" s="2" t="s">
         <v>14</v>
@@ -2076,22 +2103,22 @@
     </row>
     <row r="48" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G48" s="2" t="s">
         <v>14</v>
@@ -2102,22 +2129,22 @@
     </row>
     <row r="49" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G49" s="2" t="s">
         <v>14</v>
@@ -2128,22 +2155,22 @@
     </row>
     <row r="50" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G50" s="2" t="s">
         <v>14</v>
@@ -2154,22 +2181,22 @@
     </row>
     <row r="51" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G51" s="2" t="s">
         <v>14</v>
@@ -2180,22 +2207,22 @@
     </row>
     <row r="52" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G52" s="2" t="s">
         <v>14</v>
@@ -2206,22 +2233,22 @@
     </row>
     <row r="53" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G53" s="2" t="s">
         <v>14</v>
@@ -2232,22 +2259,22 @@
     </row>
     <row r="54" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G54" s="2" t="s">
         <v>14</v>
@@ -2258,22 +2285,22 @@
     </row>
     <row r="55" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G55" s="2" t="s">
         <v>14</v>
@@ -2284,22 +2311,22 @@
     </row>
     <row r="56" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G56" s="2" t="s">
         <v>14</v>
@@ -2310,22 +2337,22 @@
     </row>
     <row r="57" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G57" s="2" t="s">
         <v>14</v>
@@ -2336,22 +2363,22 @@
     </row>
     <row r="58" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G58" s="2" t="s">
         <v>14</v>
@@ -2362,22 +2389,22 @@
     </row>
     <row r="59" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G59" s="2" t="s">
         <v>14</v>
@@ -2388,22 +2415,22 @@
     </row>
     <row r="60" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G60" s="2" t="s">
         <v>14</v>
@@ -2414,22 +2441,22 @@
     </row>
     <row r="61" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G61" s="2" t="s">
         <v>14</v>
@@ -2440,22 +2467,22 @@
     </row>
     <row r="62" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G62" s="2" t="s">
         <v>14</v>
@@ -2466,22 +2493,22 @@
     </row>
     <row r="63" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G63" s="2" t="s">
         <v>14</v>
@@ -2492,22 +2519,22 @@
     </row>
     <row r="64" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G64" s="2" t="s">
         <v>14</v>
@@ -2518,22 +2545,22 @@
     </row>
     <row r="65" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G65" s="2" t="s">
         <v>14</v>
@@ -2544,22 +2571,22 @@
     </row>
     <row r="66" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G66" s="2" t="s">
         <v>14</v>
@@ -2570,22 +2597,22 @@
     </row>
     <row r="67" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G67" s="2" t="s">
         <v>14</v>
@@ -2596,22 +2623,22 @@
     </row>
     <row r="68" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G68" s="2" t="s">
         <v>14</v>
@@ -2622,22 +2649,22 @@
     </row>
     <row r="69" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G69" s="2" t="s">
         <v>14</v>
@@ -2648,22 +2675,22 @@
     </row>
     <row r="70" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G70" s="2" t="s">
         <v>14</v>
@@ -2674,22 +2701,22 @@
     </row>
     <row r="71" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G71" s="2" t="s">
         <v>14</v>
@@ -2700,22 +2727,22 @@
     </row>
     <row r="72" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G72" s="2" t="s">
         <v>14</v>
@@ -2726,22 +2753,22 @@
     </row>
     <row r="73" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G73" s="2" t="s">
         <v>14</v>
@@ -2752,22 +2779,22 @@
     </row>
     <row r="74" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G74" s="2" t="s">
         <v>14</v>
@@ -2778,22 +2805,22 @@
     </row>
     <row r="75" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G75" s="2" t="s">
         <v>14</v>
@@ -2804,25 +2831,25 @@
     </row>
     <row r="76" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C76" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>14</v>
+        <v>97</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F76" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G76" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H76" s="4" t="s">
         <v>15</v>
@@ -2830,25 +2857,25 @@
     </row>
     <row r="77" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C77" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>14</v>
+        <v>97</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F77" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G77" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H77" s="4" t="s">
         <v>15</v>
@@ -2856,25 +2883,25 @@
     </row>
     <row r="78" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C78" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>14</v>
+        <v>97</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F78" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G78" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H78" s="4" t="s">
         <v>15</v>
@@ -2882,25 +2909,25 @@
     </row>
     <row r="79" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C79" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>14</v>
+        <v>97</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F79" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G79" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H79" s="4" t="s">
         <v>15</v>
@@ -2908,22 +2935,22 @@
     </row>
     <row r="80" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>14</v>
+        <v>108</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F80" s="2" t="s">
-        <v>14</v>
+        <v>109</v>
       </c>
       <c r="G80" s="2" t="s">
         <v>14</v>
@@ -2934,22 +2961,22 @@
     </row>
     <row r="81" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B81" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="B81" s="2" t="s">
-        <v>104</v>
-      </c>
       <c r="C81" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>14</v>
+        <v>108</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>14</v>
+        <v>109</v>
       </c>
       <c r="G81" s="2" t="s">
         <v>14</v>
@@ -2960,22 +2987,22 @@
     </row>
     <row r="82" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C82" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B82" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>105</v>
-      </c>
       <c r="D82" s="2" t="s">
-        <v>14</v>
+        <v>108</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>14</v>
+        <v>109</v>
       </c>
       <c r="G82" s="2" t="s">
         <v>14</v>
@@ -2986,22 +3013,22 @@
     </row>
     <row r="83" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D83" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B83" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="C83" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D83" s="2" t="s">
-        <v>14</v>
-      </c>
       <c r="E83" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>14</v>
+        <v>109</v>
       </c>
       <c r="G83" s="2" t="s">
         <v>14</v>
@@ -3012,22 +3039,22 @@
     </row>
     <row r="84" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D84" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="G84" s="2" t="s">
         <v>14</v>
@@ -3038,22 +3065,22 @@
     </row>
     <row r="85" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>14</v>
+        <v>118</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="G85" s="2" t="s">
         <v>14</v>
@@ -3064,22 +3091,22 @@
     </row>
     <row r="86" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B86" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B86" s="2" t="s">
-        <v>110</v>
-      </c>
       <c r="C86" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>14</v>
+        <v>121</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="G86" s="2" t="s">
         <v>14</v>
@@ -3090,22 +3117,22 @@
     </row>
     <row r="87" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="E87" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="F87" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="B87" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="C87" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D87" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E87" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="F87" s="2" t="s">
-        <v>14</v>
       </c>
       <c r="G87" s="2" t="s">
         <v>14</v>
@@ -3116,22 +3143,22 @@
     </row>
     <row r="88" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="C88" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G88" s="2" t="s">
         <v>14</v>
@@ -3142,22 +3169,22 @@
     </row>
     <row r="89" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="C89" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G89" s="2" t="s">
         <v>14</v>
@@ -3168,22 +3195,22 @@
     </row>
     <row r="90" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="C90" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>14</v>
+        <v>133</v>
       </c>
       <c r="G90" s="2" t="s">
         <v>14</v>
@@ -3194,22 +3221,22 @@
     </row>
     <row r="91" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="C91" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>14</v>
+        <v>133</v>
       </c>
       <c r="G91" s="2" t="s">
         <v>14</v>
@@ -3220,22 +3247,22 @@
     </row>
     <row r="92" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="C92" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F92" s="2" t="s">
-        <v>14</v>
+        <v>133</v>
       </c>
       <c r="G92" s="2" t="s">
         <v>14</v>
@@ -3246,22 +3273,22 @@
     </row>
     <row r="93" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="C93" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>14</v>
+        <v>133</v>
       </c>
       <c r="G93" s="2" t="s">
         <v>14</v>
@@ -3272,19 +3299,19 @@
     </row>
     <row r="94" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="C94" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="F94" s="2" t="s">
         <v>13</v>
@@ -3298,25 +3325,25 @@
     </row>
     <row r="95" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="C95" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="F95" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H95" s="4" t="s">
         <v>15</v>
@@ -3324,25 +3351,25 @@
     </row>
     <row r="96" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="C96" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="F96" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G96" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H96" s="4" t="s">
         <v>15</v>
@@ -3350,25 +3377,25 @@
     </row>
     <row r="97" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="C97" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="F97" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H97" s="4" t="s">
         <v>15</v>
@@ -3376,25 +3403,25 @@
     </row>
     <row r="98" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="C98" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="F98" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H98" s="4" t="s">
         <v>15</v>
@@ -3402,25 +3429,25 @@
     </row>
     <row r="99" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="C99" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="F99" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H99" s="4" t="s">
         <v>15</v>
@@ -3428,19 +3455,19 @@
     </row>
     <row r="100" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="C100" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="F100" s="2" t="s">
         <v>13</v>
@@ -3454,19 +3481,19 @@
     </row>
     <row r="101" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="3" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="C101" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="F101" s="2" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Say "Details on request" once, at the foot of a painting
A work with no size or medium showed the phrase three times: as its title,
and twice more in the caption line, because the placeholder text had been
typed into the spreadsheet as well. Those 219 cells are cleared, so the site
supplies the phrase itself, once, where it belongs. The zoom panel now omits
empty Medium and Size rows rather than answering both with "On request", and
carries a single quiet note underneath instead.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Uv8R3RW9M9MhGG8c2qV64h
</commit_message>
<xml_diff>
--- a/Indus Art Collection - Catalogue.xlsx
+++ b/Indus Art Collection - Catalogue.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="149">
   <si>
     <t>ID (do not edit)</t>
   </si>
@@ -83,9 +83,6 @@
   </si>
   <si>
     <t>Gopal Naskar</t>
-  </si>
-  <si>
-    <t>Details on request</t>
   </si>
   <si>
     <t>gopal-naskar-2</t>
@@ -1046,7 +1043,7 @@
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>12</v>
@@ -1063,7 +1060,7 @@
     </row>
     <row r="8" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>23</v>
@@ -1072,7 +1069,7 @@
         <v>10</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>12</v>
@@ -1089,7 +1086,7 @@
     </row>
     <row r="9" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>23</v>
@@ -1098,7 +1095,7 @@
         <v>10</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>12</v>
@@ -1115,7 +1112,7 @@
     </row>
     <row r="10" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>23</v>
@@ -1124,7 +1121,7 @@
         <v>10</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>12</v>
@@ -1141,22 +1138,22 @@
     </row>
     <row r="11" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>14</v>
@@ -1167,22 +1164,22 @@
     </row>
     <row r="12" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>14</v>
@@ -1193,22 +1190,22 @@
     </row>
     <row r="13" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>14</v>
@@ -1219,22 +1216,22 @@
     </row>
     <row r="14" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>14</v>
@@ -1245,22 +1242,22 @@
     </row>
     <row r="15" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>14</v>
@@ -1271,22 +1268,22 @@
     </row>
     <row r="16" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>14</v>
@@ -1297,22 +1294,22 @@
     </row>
     <row r="17" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>14</v>
@@ -1323,22 +1320,22 @@
     </row>
     <row r="18" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>14</v>
@@ -1349,22 +1346,22 @@
     </row>
     <row r="19" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>14</v>
@@ -1375,22 +1372,22 @@
     </row>
     <row r="20" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>14</v>
@@ -1401,22 +1398,22 @@
     </row>
     <row r="21" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>14</v>
@@ -1427,22 +1424,22 @@
     </row>
     <row r="22" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>14</v>
@@ -1453,22 +1450,22 @@
     </row>
     <row r="23" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>14</v>
@@ -1479,22 +1476,22 @@
     </row>
     <row r="24" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>14</v>
@@ -1505,22 +1502,22 @@
     </row>
     <row r="25" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>14</v>
@@ -1531,22 +1528,22 @@
     </row>
     <row r="26" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>14</v>
@@ -1557,22 +1554,22 @@
     </row>
     <row r="27" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>14</v>
@@ -1583,22 +1580,22 @@
     </row>
     <row r="28" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>14</v>
@@ -1609,22 +1606,22 @@
     </row>
     <row r="29" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>14</v>
@@ -1635,22 +1632,22 @@
     </row>
     <row r="30" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>14</v>
@@ -1661,22 +1658,22 @@
     </row>
     <row r="31" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>14</v>
@@ -1687,22 +1684,22 @@
     </row>
     <row r="32" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>14</v>
@@ -1713,22 +1710,22 @@
     </row>
     <row r="33" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G33" s="2" t="s">
         <v>14</v>
@@ -1739,22 +1736,22 @@
     </row>
     <row r="34" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>14</v>
@@ -1765,22 +1762,22 @@
     </row>
     <row r="35" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>14</v>
@@ -1791,22 +1788,22 @@
     </row>
     <row r="36" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>14</v>
@@ -1817,22 +1814,22 @@
     </row>
     <row r="37" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>14</v>
@@ -1843,22 +1840,22 @@
     </row>
     <row r="38" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G38" s="2" t="s">
         <v>14</v>
@@ -1869,22 +1866,22 @@
     </row>
     <row r="39" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G39" s="2" t="s">
         <v>14</v>
@@ -1895,22 +1892,22 @@
     </row>
     <row r="40" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>14</v>
@@ -1921,22 +1918,22 @@
     </row>
     <row r="41" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G41" s="2" t="s">
         <v>14</v>
@@ -1947,22 +1944,22 @@
     </row>
     <row r="42" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>14</v>
@@ -1973,22 +1970,22 @@
     </row>
     <row r="43" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G43" s="2" t="s">
         <v>14</v>
@@ -1999,22 +1996,22 @@
     </row>
     <row r="44" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G44" s="2" t="s">
         <v>14</v>
@@ -2025,22 +2022,22 @@
     </row>
     <row r="45" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G45" s="2" t="s">
         <v>14</v>
@@ -2051,22 +2048,22 @@
     </row>
     <row r="46" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>14</v>
@@ -2077,22 +2074,22 @@
     </row>
     <row r="47" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G47" s="2" t="s">
         <v>14</v>
@@ -2103,22 +2100,22 @@
     </row>
     <row r="48" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G48" s="2" t="s">
         <v>14</v>
@@ -2129,22 +2126,22 @@
     </row>
     <row r="49" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G49" s="2" t="s">
         <v>14</v>
@@ -2155,22 +2152,22 @@
     </row>
     <row r="50" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G50" s="2" t="s">
         <v>14</v>
@@ -2181,22 +2178,22 @@
     </row>
     <row r="51" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G51" s="2" t="s">
         <v>14</v>
@@ -2207,22 +2204,22 @@
     </row>
     <row r="52" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G52" s="2" t="s">
         <v>14</v>
@@ -2233,22 +2230,22 @@
     </row>
     <row r="53" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G53" s="2" t="s">
         <v>14</v>
@@ -2259,22 +2256,22 @@
     </row>
     <row r="54" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G54" s="2" t="s">
         <v>14</v>
@@ -2285,22 +2282,22 @@
     </row>
     <row r="55" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G55" s="2" t="s">
         <v>14</v>
@@ -2311,22 +2308,22 @@
     </row>
     <row r="56" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G56" s="2" t="s">
         <v>14</v>
@@ -2337,22 +2334,22 @@
     </row>
     <row r="57" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G57" s="2" t="s">
         <v>14</v>
@@ -2363,22 +2360,22 @@
     </row>
     <row r="58" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G58" s="2" t="s">
         <v>14</v>
@@ -2389,22 +2386,22 @@
     </row>
     <row r="59" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G59" s="2" t="s">
         <v>14</v>
@@ -2415,22 +2412,22 @@
     </row>
     <row r="60" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G60" s="2" t="s">
         <v>14</v>
@@ -2441,22 +2438,22 @@
     </row>
     <row r="61" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G61" s="2" t="s">
         <v>14</v>
@@ -2467,22 +2464,22 @@
     </row>
     <row r="62" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G62" s="2" t="s">
         <v>14</v>
@@ -2493,22 +2490,22 @@
     </row>
     <row r="63" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G63" s="2" t="s">
         <v>14</v>
@@ -2519,22 +2516,22 @@
     </row>
     <row r="64" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G64" s="2" t="s">
         <v>14</v>
@@ -2545,22 +2542,22 @@
     </row>
     <row r="65" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G65" s="2" t="s">
         <v>14</v>
@@ -2571,22 +2568,22 @@
     </row>
     <row r="66" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G66" s="2" t="s">
         <v>14</v>
@@ -2597,22 +2594,22 @@
     </row>
     <row r="67" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G67" s="2" t="s">
         <v>14</v>
@@ -2623,22 +2620,22 @@
     </row>
     <row r="68" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G68" s="2" t="s">
         <v>14</v>
@@ -2649,22 +2646,22 @@
     </row>
     <row r="69" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G69" s="2" t="s">
         <v>14</v>
@@ -2675,22 +2672,22 @@
     </row>
     <row r="70" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G70" s="2" t="s">
         <v>14</v>
@@ -2701,22 +2698,22 @@
     </row>
     <row r="71" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G71" s="2" t="s">
         <v>14</v>
@@ -2727,22 +2724,22 @@
     </row>
     <row r="72" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G72" s="2" t="s">
         <v>14</v>
@@ -2753,22 +2750,22 @@
     </row>
     <row r="73" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G73" s="2" t="s">
         <v>14</v>
@@ -2779,22 +2776,22 @@
     </row>
     <row r="74" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G74" s="2" t="s">
         <v>14</v>
@@ -2805,22 +2802,22 @@
     </row>
     <row r="75" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G75" s="2" t="s">
         <v>14</v>
@@ -2831,25 +2828,25 @@
     </row>
     <row r="76" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B76" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="B76" s="2" t="s">
-        <v>96</v>
       </c>
       <c r="C76" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D76" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E76" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="E76" s="2" t="s">
-        <v>98</v>
       </c>
       <c r="F76" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G76" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H76" s="4" t="s">
         <v>15</v>
@@ -2857,25 +2854,25 @@
     </row>
     <row r="77" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C77" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D77" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E77" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="E77" s="2" t="s">
-        <v>98</v>
       </c>
       <c r="F77" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G77" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H77" s="4" t="s">
         <v>15</v>
@@ -2883,25 +2880,25 @@
     </row>
     <row r="78" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C78" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F78" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G78" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H78" s="4" t="s">
         <v>15</v>
@@ -2909,25 +2906,25 @@
     </row>
     <row r="79" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C79" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F79" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G79" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H79" s="4" t="s">
         <v>15</v>
@@ -2935,22 +2932,22 @@
     </row>
     <row r="80" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B80" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B80" s="2" t="s">
+      <c r="C80" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C80" s="2" t="s">
+      <c r="D80" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="D80" s="2" t="s">
+      <c r="E80" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="E80" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F80" s="2" t="s">
-        <v>109</v>
       </c>
       <c r="G80" s="2" t="s">
         <v>14</v>
@@ -2961,22 +2958,22 @@
     </row>
     <row r="81" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B81" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C81" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C81" s="2" t="s">
+      <c r="D81" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="D81" s="2" t="s">
+      <c r="E81" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F81" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="E81" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F81" s="2" t="s">
-        <v>109</v>
       </c>
       <c r="G81" s="2" t="s">
         <v>14</v>
@@ -2987,22 +2984,22 @@
     </row>
     <row r="82" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B82" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C82" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C82" s="2" t="s">
+      <c r="D82" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="D82" s="2" t="s">
+      <c r="E82" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="E82" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F82" s="2" t="s">
-        <v>109</v>
       </c>
       <c r="G82" s="2" t="s">
         <v>14</v>
@@ -3013,22 +3010,22 @@
     </row>
     <row r="83" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B83" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C83" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C83" s="2" t="s">
+      <c r="D83" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="D83" s="2" t="s">
+      <c r="E83" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="E83" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F83" s="2" t="s">
-        <v>109</v>
       </c>
       <c r="G83" s="2" t="s">
         <v>14</v>
@@ -3039,22 +3036,22 @@
     </row>
     <row r="84" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B84" s="2" t="s">
+      <c r="C84" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E84" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="C84" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="D84" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E84" s="2" t="s">
+      <c r="F84" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="F84" s="2" t="s">
-        <v>116</v>
       </c>
       <c r="G84" s="2" t="s">
         <v>14</v>
@@ -3065,22 +3062,22 @@
     </row>
     <row r="85" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D85" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="B85" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="C85" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="D85" s="2" t="s">
+      <c r="E85" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="E85" s="2" t="s">
-        <v>119</v>
-      </c>
       <c r="F85" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G85" s="2" t="s">
         <v>14</v>
@@ -3091,22 +3088,22 @@
     </row>
     <row r="86" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D86" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B86" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="C86" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="D86" s="2" t="s">
+      <c r="E86" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="E86" s="2" t="s">
-        <v>122</v>
-      </c>
       <c r="F86" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G86" s="2" t="s">
         <v>14</v>
@@ -3117,22 +3114,22 @@
     </row>
     <row r="87" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D87" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="B87" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="C87" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="D87" s="2" t="s">
+      <c r="E87" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="E87" s="2" t="s">
-        <v>125</v>
-      </c>
       <c r="F87" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G87" s="2" t="s">
         <v>14</v>
@@ -3143,19 +3140,19 @@
     </row>
     <row r="88" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B88" s="2" t="s">
         <v>126</v>
-      </c>
-      <c r="B88" s="2" t="s">
-        <v>127</v>
       </c>
       <c r="C88" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F88" s="2" t="s">
         <v>13</v>
@@ -3169,19 +3166,19 @@
     </row>
     <row r="89" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C89" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F89" s="2" t="s">
         <v>13</v>
@@ -3195,22 +3192,22 @@
     </row>
     <row r="90" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="B90" s="2" t="s">
         <v>131</v>
-      </c>
-      <c r="B90" s="2" t="s">
-        <v>132</v>
       </c>
       <c r="C90" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G90" s="2" t="s">
         <v>14</v>
@@ -3221,22 +3218,22 @@
     </row>
     <row r="91" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C91" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G91" s="2" t="s">
         <v>14</v>
@@ -3247,22 +3244,22 @@
     </row>
     <row r="92" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C92" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F92" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G92" s="2" t="s">
         <v>14</v>
@@ -3273,22 +3270,22 @@
     </row>
     <row r="93" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C93" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G93" s="2" t="s">
         <v>14</v>
@@ -3299,19 +3296,19 @@
     </row>
     <row r="94" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="B94" s="2" t="s">
         <v>137</v>
-      </c>
-      <c r="B94" s="2" t="s">
-        <v>138</v>
       </c>
       <c r="C94" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F94" s="2" t="s">
         <v>13</v>
@@ -3325,25 +3322,25 @@
     </row>
     <row r="95" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C95" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F95" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H95" s="4" t="s">
         <v>15</v>
@@ -3351,25 +3348,25 @@
     </row>
     <row r="96" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C96" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F96" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G96" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H96" s="4" t="s">
         <v>15</v>
@@ -3377,25 +3374,25 @@
     </row>
     <row r="97" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C97" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F97" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H97" s="4" t="s">
         <v>15</v>
@@ -3403,25 +3400,25 @@
     </row>
     <row r="98" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C98" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F98" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H98" s="4" t="s">
         <v>15</v>
@@ -3429,25 +3426,25 @@
     </row>
     <row r="99" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C99" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F99" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H99" s="4" t="s">
         <v>15</v>
@@ -3455,19 +3452,19 @@
     </row>
     <row r="100" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C100" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D100" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E100" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="E100" s="2" t="s">
-        <v>148</v>
       </c>
       <c r="F100" s="2" t="s">
         <v>13</v>
@@ -3481,19 +3478,19 @@
     </row>
     <row r="101" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C101" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D101" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E101" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="E101" s="2" t="s">
-        <v>148</v>
       </c>
       <c r="F101" s="2" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Identify paintings by reference number instead of artist name
The website no longer names any painter. Each work carries a reference
(IAC-001 …) under its thumbnail, in the enlarged view and in the enquiry
it starts, and the image files are named after the reference so no name
can be read out of the page source either.

Removed with it: the Meet the artists button, the Artists tab and the
artist pages (old links land on the gallery), and the artwork under
"The painters we represent", which is now text only.

Which painter each reference belongs to is recorded in the catalogue
spreadsheet and in Painting Reference List.md, neither of them published.
scripts/refs.json pins a reference to its photograph for good, so a
number quoted to a customer always means the same painting.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Uv8R3RW9M9MhGG8c2qV64h
</commit_message>
<xml_diff>
--- a/Indus Art Collection - Catalogue.xlsx
+++ b/Indus Art Collection - Catalogue.xlsx
@@ -13,7 +13,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="149">
   <si>
-    <t>ID (do not edit)</t>
+    <t>Reference (do not edit)</t>
   </si>
   <si>
     <t>Artist (do not edit)</t>
@@ -37,64 +37,190 @@
     <t>Description (editable)</t>
   </si>
   <si>
-    <t>ashok-rathod-painting-1</t>
+    <t>IAC-001</t>
+  </si>
+  <si>
+    <t>Umesh Kumar Saxena</t>
+  </si>
+  <si>
+    <t>Contemporary</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>70 x 70 in / 178 x 178 cm</t>
+  </si>
+  <si>
+    <t>Acrylic on canvas</t>
+  </si>
+  <si>
+    <t>Add a short description of this painting here.</t>
+  </si>
+  <si>
+    <t>IAC-002</t>
+  </si>
+  <si>
+    <t>36 x 72 in</t>
+  </si>
+  <si>
+    <t>2025</t>
+  </si>
+  <si>
+    <t>IAC-003</t>
+  </si>
+  <si>
+    <t>IAC-004</t>
+  </si>
+  <si>
+    <t>IAC-005</t>
+  </si>
+  <si>
+    <t>IAC-006</t>
+  </si>
+  <si>
+    <t>IAC-007</t>
+  </si>
+  <si>
+    <t>Triptych</t>
+  </si>
+  <si>
+    <t>18 x 60 in each</t>
+  </si>
+  <si>
+    <t>IAC-008</t>
+  </si>
+  <si>
+    <t>IAC-009</t>
+  </si>
+  <si>
+    <t>Kandan G</t>
+  </si>
+  <si>
+    <t>Banaras Series</t>
+  </si>
+  <si>
+    <t>24 x 48 in / 61 x 122 cm</t>
+  </si>
+  <si>
+    <t>2024</t>
+  </si>
+  <si>
+    <t>IAC-010</t>
+  </si>
+  <si>
+    <t>IAC-011</t>
+  </si>
+  <si>
+    <t>36 x 60 in / 92 x 153 cm</t>
+  </si>
+  <si>
+    <t>IAC-012</t>
+  </si>
+  <si>
+    <t>IAC-013</t>
+  </si>
+  <si>
+    <t>Nirakar Chowdhury</t>
+  </si>
+  <si>
+    <t>140 x 85 cm</t>
+  </si>
+  <si>
+    <t>IAC-014</t>
+  </si>
+  <si>
+    <t>153 x 191 cm</t>
+  </si>
+  <si>
+    <t>IAC-015</t>
   </si>
   <si>
     <t>Ashok Rathod</t>
   </si>
   <si>
-    <t>Contemporary</t>
-  </si>
-  <si>
     <t>Nandi</t>
   </si>
   <si>
     <t>24 x 24 in</t>
   </si>
   <si>
-    <t>Acrylic on canvas</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Add a short description of this painting here.</t>
-  </si>
-  <si>
-    <t>ashok-rathod-painting-2</t>
+    <t>IAC-016</t>
   </si>
   <si>
     <t>36 x 60 in</t>
   </si>
   <si>
-    <t>ashok-rathod-painting-3</t>
-  </si>
-  <si>
-    <t>ashok-rathod-painting-4</t>
-  </si>
-  <si>
-    <t>ashok-rathod-painting-5</t>
+    <t>IAC-017</t>
+  </si>
+  <si>
+    <t>IAC-018</t>
+  </si>
+  <si>
+    <t>IAC-019</t>
   </si>
   <si>
     <t>48 x 72 in</t>
   </si>
   <si>
-    <t>gopal-naskar-1</t>
+    <t>IAC-020</t>
   </si>
   <si>
     <t>Gopal Naskar</t>
   </si>
   <si>
-    <t>gopal-naskar-2</t>
-  </si>
-  <si>
-    <t>gopal-naskar-3</t>
-  </si>
-  <si>
-    <t>gopal-naskar-4</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-10</t>
+    <t>IAC-021</t>
+  </si>
+  <si>
+    <t>IAC-022</t>
+  </si>
+  <si>
+    <t>IAC-023</t>
+  </si>
+  <si>
+    <t>IAC-024</t>
+  </si>
+  <si>
+    <t>Umendra P. Singh</t>
+  </si>
+  <si>
+    <t>Oil on Canvas</t>
+  </si>
+  <si>
+    <t>IAC-025</t>
+  </si>
+  <si>
+    <t>IAC-026</t>
+  </si>
+  <si>
+    <t>IAC-027</t>
+  </si>
+  <si>
+    <t>IAC-028</t>
+  </si>
+  <si>
+    <t>M. Salim</t>
+  </si>
+  <si>
+    <t>Traditional</t>
+  </si>
+  <si>
+    <t>Landscape</t>
+  </si>
+  <si>
+    <t>Mix Medium</t>
+  </si>
+  <si>
+    <t>IAC-029</t>
+  </si>
+  <si>
+    <t>IAC-030</t>
+  </si>
+  <si>
+    <t>IAC-031</t>
+  </si>
+  <si>
+    <t>IAC-032</t>
   </si>
   <si>
     <t>Folk &amp; Tribal Masters</t>
@@ -103,253 +229,199 @@
     <t>Folk</t>
   </si>
   <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-13</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-14</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-15</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-16</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-17</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-18</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-19</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-24</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-26</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-27</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-28</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-29</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-31</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-32</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-33</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-36</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-38</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-39</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-40</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-41</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-42</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-43</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-44</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-45</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-46</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-47</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-48</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-49</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-50</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-51</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-53</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-54</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-55</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-57</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-59</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-60</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-61</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-62</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-64</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-65</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-66</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-67</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-68</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-70</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-72</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-73</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-74</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-75</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-76</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-77</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-78</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-79</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-80</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-81</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-83</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-85</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-86</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-87</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-88</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-89</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-90</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-91</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-92</t>
-  </si>
-  <si>
-    <t>india-folk-tribal-paintings-song-collection-2604-260408-001807-93</t>
-  </si>
-  <si>
-    <t>kandan-g-1</t>
-  </si>
-  <si>
-    <t>Kandan G</t>
-  </si>
-  <si>
-    <t>Banaras Series</t>
-  </si>
-  <si>
-    <t>24 x 48 in / 61 x 122 cm</t>
-  </si>
-  <si>
-    <t>2024</t>
-  </si>
-  <si>
-    <t>kandan-g-2</t>
-  </si>
-  <si>
-    <t>kandan-g-3</t>
-  </si>
-  <si>
-    <t>36 x 60 in / 92 x 153 cm</t>
-  </si>
-  <si>
-    <t>2025</t>
-  </si>
-  <si>
-    <t>kandan-g-4</t>
-  </si>
-  <si>
-    <t>m-salim-painting-1</t>
-  </si>
-  <si>
-    <t>M. Salim</t>
-  </si>
-  <si>
-    <t>Traditional</t>
-  </si>
-  <si>
-    <t>Landscape</t>
-  </si>
-  <si>
-    <t>Mix Medium</t>
-  </si>
-  <si>
-    <t>m-salim-painting-2</t>
-  </si>
-  <si>
-    <t>m-salim-painting-3</t>
-  </si>
-  <si>
-    <t>m-salim-painting-4</t>
-  </si>
-  <si>
-    <t>n-k-mishra-1</t>
+    <t>IAC-033</t>
+  </si>
+  <si>
+    <t>IAC-034</t>
+  </si>
+  <si>
+    <t>IAC-035</t>
+  </si>
+  <si>
+    <t>IAC-036</t>
+  </si>
+  <si>
+    <t>IAC-037</t>
+  </si>
+  <si>
+    <t>IAC-038</t>
+  </si>
+  <si>
+    <t>IAC-039</t>
+  </si>
+  <si>
+    <t>IAC-040</t>
+  </si>
+  <si>
+    <t>IAC-041</t>
+  </si>
+  <si>
+    <t>IAC-042</t>
+  </si>
+  <si>
+    <t>IAC-043</t>
+  </si>
+  <si>
+    <t>IAC-044</t>
+  </si>
+  <si>
+    <t>IAC-045</t>
+  </si>
+  <si>
+    <t>IAC-046</t>
+  </si>
+  <si>
+    <t>IAC-047</t>
+  </si>
+  <si>
+    <t>IAC-048</t>
+  </si>
+  <si>
+    <t>IAC-049</t>
+  </si>
+  <si>
+    <t>IAC-050</t>
+  </si>
+  <si>
+    <t>IAC-051</t>
+  </si>
+  <si>
+    <t>IAC-052</t>
+  </si>
+  <si>
+    <t>IAC-053</t>
+  </si>
+  <si>
+    <t>IAC-054</t>
+  </si>
+  <si>
+    <t>IAC-055</t>
+  </si>
+  <si>
+    <t>IAC-056</t>
+  </si>
+  <si>
+    <t>IAC-057</t>
+  </si>
+  <si>
+    <t>IAC-058</t>
+  </si>
+  <si>
+    <t>IAC-059</t>
+  </si>
+  <si>
+    <t>IAC-060</t>
+  </si>
+  <si>
+    <t>IAC-061</t>
+  </si>
+  <si>
+    <t>IAC-062</t>
+  </si>
+  <si>
+    <t>IAC-063</t>
+  </si>
+  <si>
+    <t>IAC-064</t>
+  </si>
+  <si>
+    <t>IAC-065</t>
+  </si>
+  <si>
+    <t>IAC-066</t>
+  </si>
+  <si>
+    <t>IAC-067</t>
+  </si>
+  <si>
+    <t>IAC-068</t>
+  </si>
+  <si>
+    <t>IAC-069</t>
+  </si>
+  <si>
+    <t>IAC-070</t>
+  </si>
+  <si>
+    <t>IAC-071</t>
+  </si>
+  <si>
+    <t>IAC-072</t>
+  </si>
+  <si>
+    <t>IAC-073</t>
+  </si>
+  <si>
+    <t>IAC-074</t>
+  </si>
+  <si>
+    <t>IAC-075</t>
+  </si>
+  <si>
+    <t>IAC-076</t>
+  </si>
+  <si>
+    <t>IAC-077</t>
+  </si>
+  <si>
+    <t>IAC-078</t>
+  </si>
+  <si>
+    <t>IAC-079</t>
+  </si>
+  <si>
+    <t>IAC-080</t>
+  </si>
+  <si>
+    <t>IAC-081</t>
+  </si>
+  <si>
+    <t>IAC-082</t>
+  </si>
+  <si>
+    <t>IAC-083</t>
+  </si>
+  <si>
+    <t>IAC-084</t>
+  </si>
+  <si>
+    <t>IAC-085</t>
+  </si>
+  <si>
+    <t>IAC-086</t>
+  </si>
+  <si>
+    <t>IAC-087</t>
+  </si>
+  <si>
+    <t>IAC-088</t>
+  </si>
+  <si>
+    <t>IAC-089</t>
+  </si>
+  <si>
+    <t>IAC-090</t>
+  </si>
+  <si>
+    <t>IAC-091</t>
+  </si>
+  <si>
+    <t>IAC-092</t>
+  </si>
+  <si>
+    <t>IAC-093</t>
+  </si>
+  <si>
+    <t>IAC-094</t>
+  </si>
+  <si>
+    <t>IAC-095</t>
+  </si>
+  <si>
+    <t>IAC-096</t>
+  </si>
+  <si>
+    <t>IAC-097</t>
   </si>
   <si>
     <t>N. K. Mishra</t>
@@ -361,7 +433,7 @@
     <t>Water colour and gouache on paper</t>
   </si>
   <si>
-    <t>n-k-mishra-2</t>
+    <t>IAC-098</t>
   </si>
   <si>
     <t>Parvati and Ganesha</t>
@@ -370,7 +442,7 @@
     <t>13.2 x 7.1 in</t>
   </si>
   <si>
-    <t>n-k-mishra-3</t>
+    <t>IAC-099</t>
   </si>
   <si>
     <t>Ganesh</t>
@@ -379,85 +451,13 @@
     <t>12.5 x 8.5 in</t>
   </si>
   <si>
-    <t>n-k-mishra-4</t>
+    <t>IAC-100</t>
   </si>
   <si>
     <t>Hanuman</t>
   </si>
   <si>
     <t>19.5 x 19.5 in</t>
-  </si>
-  <si>
-    <t>nirakaar-chaudhary-painting-1</t>
-  </si>
-  <si>
-    <t>Nirakar Chowdhury</t>
-  </si>
-  <si>
-    <t>140 x 85 cm</t>
-  </si>
-  <si>
-    <t>nirakaar-chaudhary-painting-2</t>
-  </si>
-  <si>
-    <t>153 x 191 cm</t>
-  </si>
-  <si>
-    <t>umendra-p-singh-1</t>
-  </si>
-  <si>
-    <t>Umendra P. Singh</t>
-  </si>
-  <si>
-    <t>Oil on Canvas</t>
-  </si>
-  <si>
-    <t>umendra-p-singh-2</t>
-  </si>
-  <si>
-    <t>umendra-p-singh-3</t>
-  </si>
-  <si>
-    <t>umendra-p-singh-4</t>
-  </si>
-  <si>
-    <t>umesh-ji-1</t>
-  </si>
-  <si>
-    <t>Umesh Kumar Saxena</t>
-  </si>
-  <si>
-    <t>70 x 70 in / 178 x 178 cm</t>
-  </si>
-  <si>
-    <t>umesh-ji-2</t>
-  </si>
-  <si>
-    <t>36 x 72 in</t>
-  </si>
-  <si>
-    <t>umesh-ji-3</t>
-  </si>
-  <si>
-    <t>umesh-ji-4</t>
-  </si>
-  <si>
-    <t>umesh-ji-5</t>
-  </si>
-  <si>
-    <t>umesh-ji-6</t>
-  </si>
-  <si>
-    <t>umesh-kumar-saxena-painting-1-1</t>
-  </si>
-  <si>
-    <t>Triptych</t>
-  </si>
-  <si>
-    <t>18 x 60 in each</t>
-  </si>
-  <si>
-    <t>umesh-kumar-saxena-painting-1-2</t>
   </si>
 </sst>
 </file>
@@ -477,8 +477,7 @@
       <color rgb="FFFFFFFF"/>
     </font>
     <font>
-      <color rgb="FF999999"/>
-      <sz val="9"/>
+      <b/>
     </font>
     <font>
       <i/>
@@ -866,7 +865,7 @@
   <dimension ref="A1:H101"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="46" customWidth="1"/>
+    <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
@@ -922,15 +921,15 @@
         <v>13</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>9</v>
@@ -942,16 +941,16 @@
         <v>11</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -968,16 +967,16 @@
         <v>11</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -994,16 +993,16 @@
         <v>11</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1020,68 +1019,68 @@
         <v>11</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1089,25 +1088,25 @@
         <v>25</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1115,2391 +1114,2391 @@
         <v>26</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C11" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>14</v>
-      </c>
       <c r="F11" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>14</v>
-      </c>
       <c r="E12" s="2" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>14</v>
-      </c>
       <c r="E13" s="2" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>14</v>
+        <v>49</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="25" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>28</v>
+        <v>56</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>14</v>
+        <v>57</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="26" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>28</v>
+        <v>56</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>14</v>
+        <v>57</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="27" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>28</v>
+        <v>56</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>14</v>
+        <v>57</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="28" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>46</v>
+        <v>60</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>28</v>
+        <v>56</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>14</v>
+        <v>57</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="29" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>28</v>
+        <v>62</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>14</v>
+        <v>64</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>14</v>
+        <v>65</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="30" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>28</v>
+        <v>62</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>14</v>
+        <v>64</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>14</v>
+        <v>65</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="31" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>28</v>
+        <v>62</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>14</v>
+        <v>64</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>14</v>
+        <v>65</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="32" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>28</v>
+        <v>62</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>14</v>
+        <v>64</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>14</v>
+        <v>65</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="33" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="34" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="35" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="36" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="37" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="38" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="39" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="40" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="41" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>59</v>
+        <v>79</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H41" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="42" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="43" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>61</v>
+        <v>81</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="44" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="45" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>63</v>
+        <v>83</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="46" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>64</v>
+        <v>84</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="47" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="48" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="49" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>67</v>
+        <v>87</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="50" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>68</v>
+        <v>88</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="51" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="52" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="53" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H53" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="54" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H54" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="55" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H55" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="56" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="57" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H57" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="58" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H58" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="59" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H59" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="60" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
-        <v>78</v>
+        <v>98</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="61" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G61" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H61" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="62" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H62" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="63" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
-        <v>81</v>
+        <v>101</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H63" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="64" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>82</v>
+        <v>102</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G64" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H64" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="65" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="66" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>84</v>
+        <v>104</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H66" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="67" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
-        <v>85</v>
+        <v>105</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H67" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="68" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>86</v>
+        <v>106</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G68" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H68" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="69" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
-        <v>87</v>
+        <v>107</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H69" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="70" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
-        <v>88</v>
+        <v>108</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H70" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="71" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
-        <v>89</v>
+        <v>109</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H71" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="72" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H72" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="73" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
-        <v>91</v>
+        <v>111</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H73" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="74" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H74" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="75" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
-        <v>93</v>
+        <v>113</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H75" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="76" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
-        <v>94</v>
+        <v>114</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>96</v>
+        <v>11</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>97</v>
+        <v>11</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G76" s="2" t="s">
-        <v>98</v>
+        <v>11</v>
       </c>
       <c r="H76" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="77" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>96</v>
+        <v>11</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>97</v>
+        <v>11</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G77" s="2" t="s">
-        <v>98</v>
+        <v>11</v>
       </c>
       <c r="H77" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="78" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>96</v>
+        <v>11</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>101</v>
+        <v>11</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G78" s="2" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
       <c r="H78" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="79" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>96</v>
+        <v>11</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>101</v>
+        <v>11</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G79" s="2" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
       <c r="H79" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="80" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>107</v>
+        <v>11</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F80" s="2" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
       <c r="G80" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H80" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="81" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>107</v>
+        <v>11</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
       <c r="G81" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H81" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="82" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>107</v>
+        <v>11</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
       <c r="G82" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H82" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="83" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>107</v>
+        <v>11</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
       <c r="G83" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H83" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="84" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>113</v>
+        <v>70</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>114</v>
+        <v>11</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>115</v>
+        <v>11</v>
       </c>
       <c r="G84" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H84" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="85" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>113</v>
+        <v>70</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>117</v>
+        <v>11</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>118</v>
+        <v>11</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>115</v>
+        <v>11</v>
       </c>
       <c r="G85" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H85" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="86" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>113</v>
+        <v>70</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>120</v>
+        <v>11</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>121</v>
+        <v>11</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>115</v>
+        <v>11</v>
       </c>
       <c r="G86" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H86" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="87" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>113</v>
+        <v>70</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>123</v>
+        <v>11</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>124</v>
+        <v>11</v>
       </c>
       <c r="F87" s="2" t="s">
-        <v>115</v>
+        <v>11</v>
       </c>
       <c r="G87" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H87" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="88" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>126</v>
+        <v>70</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>127</v>
+        <v>11</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G88" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H88" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="89" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>126</v>
+        <v>70</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>129</v>
+        <v>11</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G89" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H89" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="90" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>131</v>
+        <v>70</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>132</v>
+        <v>11</v>
       </c>
       <c r="G90" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H90" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="91" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>131</v>
+        <v>70</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>132</v>
+        <v>11</v>
       </c>
       <c r="G91" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H91" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="92" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>131</v>
+        <v>70</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F92" s="2" t="s">
-        <v>132</v>
+        <v>11</v>
       </c>
       <c r="G92" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H92" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="93" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>131</v>
+        <v>70</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>132</v>
+        <v>11</v>
       </c>
       <c r="G93" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H93" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="94" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>137</v>
+        <v>70</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>138</v>
+        <v>11</v>
       </c>
       <c r="F94" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H94" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="95" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>137</v>
+        <v>70</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>140</v>
+        <v>11</v>
       </c>
       <c r="F95" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
       <c r="H95" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="96" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>137</v>
+        <v>70</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>140</v>
+        <v>11</v>
       </c>
       <c r="F96" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G96" s="2" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
       <c r="H96" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="97" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>137</v>
+        <v>70</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>140</v>
+        <v>11</v>
       </c>
       <c r="F97" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
       <c r="H97" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="98" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="B98" s="2" t="s">
         <v>137</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="F98" s="2" t="s">
-        <v>13</v>
+        <v>139</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
       <c r="H98" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="99" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B99" s="2" t="s">
         <v>137</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>14</v>
+        <v>141</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F99" s="2" t="s">
-        <v>13</v>
+        <v>139</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
       <c r="H99" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="100" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>137</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F100" s="2" t="s">
-        <v>13</v>
+        <v>139</v>
       </c>
       <c r="G100" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H100" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="101" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>137</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F101" s="2" t="s">
-        <v>13</v>
+        <v>139</v>
       </c>
       <c r="G101" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H101" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add M. D. Ishak's 67 landscapes to the collection
Extracted from "pdf M.d ishak paintings 66.pdf" and hung directly after
IAC-014, as asked. They take references IAC-101 to IAC-167: a reference
already given out must keep meaning the same painting, so the numbers
carry on from the end rather than renumbering the collection.

Eight of the photographs show the work in its frame and mount. Those are
now cropped to the painting itself by findFrameBox, which tells frame
from painting by flatness rather than colour — a black frame and a
black-grounded canvas are the same colour, but only one of them has
texture. It runs solely on the photographs listed in FRAMED.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Uv8R3RW9M9MhGG8c2qV64h
</commit_message>
<xml_diff>
--- a/Indus Art Collection - Catalogue.xlsx
+++ b/Indus Art Collection - Catalogue.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1344" uniqueCount="217">
   <si>
     <t>Reference (do not edit)</t>
   </si>
@@ -133,6 +133,213 @@
     <t>153 x 191 cm</t>
   </si>
   <si>
+    <t>IAC-101</t>
+  </si>
+  <si>
+    <t>M. D. Ishak</t>
+  </si>
+  <si>
+    <t>Traditional</t>
+  </si>
+  <si>
+    <t>IAC-102</t>
+  </si>
+  <si>
+    <t>IAC-103</t>
+  </si>
+  <si>
+    <t>IAC-104</t>
+  </si>
+  <si>
+    <t>IAC-105</t>
+  </si>
+  <si>
+    <t>IAC-106</t>
+  </si>
+  <si>
+    <t>IAC-107</t>
+  </si>
+  <si>
+    <t>IAC-108</t>
+  </si>
+  <si>
+    <t>IAC-109</t>
+  </si>
+  <si>
+    <t>IAC-110</t>
+  </si>
+  <si>
+    <t>IAC-111</t>
+  </si>
+  <si>
+    <t>IAC-112</t>
+  </si>
+  <si>
+    <t>IAC-113</t>
+  </si>
+  <si>
+    <t>IAC-114</t>
+  </si>
+  <si>
+    <t>IAC-115</t>
+  </si>
+  <si>
+    <t>IAC-116</t>
+  </si>
+  <si>
+    <t>IAC-117</t>
+  </si>
+  <si>
+    <t>IAC-118</t>
+  </si>
+  <si>
+    <t>IAC-119</t>
+  </si>
+  <si>
+    <t>IAC-120</t>
+  </si>
+  <si>
+    <t>IAC-121</t>
+  </si>
+  <si>
+    <t>IAC-122</t>
+  </si>
+  <si>
+    <t>IAC-123</t>
+  </si>
+  <si>
+    <t>IAC-124</t>
+  </si>
+  <si>
+    <t>IAC-125</t>
+  </si>
+  <si>
+    <t>IAC-126</t>
+  </si>
+  <si>
+    <t>IAC-127</t>
+  </si>
+  <si>
+    <t>IAC-128</t>
+  </si>
+  <si>
+    <t>IAC-129</t>
+  </si>
+  <si>
+    <t>IAC-130</t>
+  </si>
+  <si>
+    <t>IAC-131</t>
+  </si>
+  <si>
+    <t>IAC-132</t>
+  </si>
+  <si>
+    <t>IAC-133</t>
+  </si>
+  <si>
+    <t>IAC-134</t>
+  </si>
+  <si>
+    <t>IAC-135</t>
+  </si>
+  <si>
+    <t>IAC-136</t>
+  </si>
+  <si>
+    <t>IAC-137</t>
+  </si>
+  <si>
+    <t>IAC-138</t>
+  </si>
+  <si>
+    <t>IAC-139</t>
+  </si>
+  <si>
+    <t>IAC-140</t>
+  </si>
+  <si>
+    <t>IAC-141</t>
+  </si>
+  <si>
+    <t>IAC-142</t>
+  </si>
+  <si>
+    <t>IAC-143</t>
+  </si>
+  <si>
+    <t>IAC-144</t>
+  </si>
+  <si>
+    <t>IAC-145</t>
+  </si>
+  <si>
+    <t>IAC-146</t>
+  </si>
+  <si>
+    <t>IAC-147</t>
+  </si>
+  <si>
+    <t>IAC-148</t>
+  </si>
+  <si>
+    <t>IAC-149</t>
+  </si>
+  <si>
+    <t>IAC-150</t>
+  </si>
+  <si>
+    <t>IAC-151</t>
+  </si>
+  <si>
+    <t>IAC-152</t>
+  </si>
+  <si>
+    <t>IAC-153</t>
+  </si>
+  <si>
+    <t>IAC-154</t>
+  </si>
+  <si>
+    <t>IAC-155</t>
+  </si>
+  <si>
+    <t>IAC-156</t>
+  </si>
+  <si>
+    <t>IAC-157</t>
+  </si>
+  <si>
+    <t>IAC-158</t>
+  </si>
+  <si>
+    <t>IAC-159</t>
+  </si>
+  <si>
+    <t>IAC-160</t>
+  </si>
+  <si>
+    <t>IAC-161</t>
+  </si>
+  <si>
+    <t>IAC-162</t>
+  </si>
+  <si>
+    <t>IAC-163</t>
+  </si>
+  <si>
+    <t>IAC-164</t>
+  </si>
+  <si>
+    <t>IAC-165</t>
+  </si>
+  <si>
+    <t>IAC-166</t>
+  </si>
+  <si>
+    <t>IAC-167</t>
+  </si>
+  <si>
     <t>IAC-015</t>
   </si>
   <si>
@@ -200,9 +407,6 @@
   </si>
   <si>
     <t>M. Salim</t>
-  </si>
-  <si>
-    <t>Traditional</t>
   </si>
   <si>
     <t>Landscape</t>
@@ -862,7 +1066,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H101"/>
+  <dimension ref="A1:H168"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1273,16 +1477,16 @@
         <v>41</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>11</v>
@@ -1293,22 +1497,22 @@
     </row>
     <row r="17" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>11</v>
@@ -1319,22 +1523,22 @@
     </row>
     <row r="18" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>11</v>
@@ -1345,22 +1549,22 @@
     </row>
     <row r="19" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>11</v>
@@ -1371,22 +1575,22 @@
     </row>
     <row r="20" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>11</v>
@@ -1397,22 +1601,22 @@
     </row>
     <row r="21" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>11</v>
@@ -1423,22 +1627,22 @@
     </row>
     <row r="22" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>11</v>
@@ -1449,22 +1653,22 @@
     </row>
     <row r="23" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>11</v>
@@ -1475,22 +1679,22 @@
     </row>
     <row r="24" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>11</v>
@@ -1501,13 +1705,13 @@
     </row>
     <row r="25" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>11</v>
@@ -1516,7 +1720,7 @@
         <v>11</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>11</v>
@@ -1527,13 +1731,13 @@
     </row>
     <row r="26" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>11</v>
@@ -1542,7 +1746,7 @@
         <v>11</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>11</v>
@@ -1553,13 +1757,13 @@
     </row>
     <row r="27" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>11</v>
@@ -1568,7 +1772,7 @@
         <v>11</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>11</v>
@@ -1579,13 +1783,13 @@
     </row>
     <row r="28" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>11</v>
@@ -1594,7 +1798,7 @@
         <v>11</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>11</v>
@@ -1605,22 +1809,22 @@
     </row>
     <row r="29" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>64</v>
+        <v>11</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>11</v>
@@ -1631,22 +1835,22 @@
     </row>
     <row r="30" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>64</v>
+        <v>11</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>11</v>
@@ -1657,22 +1861,22 @@
     </row>
     <row r="31" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>64</v>
+        <v>11</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>11</v>
@@ -1683,22 +1887,22 @@
     </row>
     <row r="32" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>64</v>
+        <v>11</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>11</v>
@@ -1709,13 +1913,13 @@
     </row>
     <row r="33" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>11</v>
@@ -1735,13 +1939,13 @@
     </row>
     <row r="34" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>11</v>
@@ -1761,13 +1965,13 @@
     </row>
     <row r="35" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>11</v>
@@ -1787,13 +1991,13 @@
     </row>
     <row r="36" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>11</v>
@@ -1813,13 +2017,13 @@
     </row>
     <row r="37" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>11</v>
@@ -1839,13 +2043,13 @@
     </row>
     <row r="38" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>11</v>
@@ -1865,13 +2069,13 @@
     </row>
     <row r="39" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>11</v>
@@ -1891,13 +2095,13 @@
     </row>
     <row r="40" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>11</v>
@@ -1917,13 +2121,13 @@
     </row>
     <row r="41" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>11</v>
@@ -1943,13 +2147,13 @@
     </row>
     <row r="42" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>11</v>
@@ -1969,13 +2173,13 @@
     </row>
     <row r="43" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>11</v>
@@ -1995,13 +2199,13 @@
     </row>
     <row r="44" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>11</v>
@@ -2021,13 +2225,13 @@
     </row>
     <row r="45" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>11</v>
@@ -2047,13 +2251,13 @@
     </row>
     <row r="46" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>11</v>
@@ -2073,13 +2277,13 @@
     </row>
     <row r="47" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>11</v>
@@ -2099,13 +2303,13 @@
     </row>
     <row r="48" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>11</v>
@@ -2125,13 +2329,13 @@
     </row>
     <row r="49" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>11</v>
@@ -2151,13 +2355,13 @@
     </row>
     <row r="50" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>11</v>
@@ -2177,13 +2381,13 @@
     </row>
     <row r="51" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>11</v>
@@ -2203,13 +2407,13 @@
     </row>
     <row r="52" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>11</v>
@@ -2229,13 +2433,13 @@
     </row>
     <row r="53" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>11</v>
@@ -2255,13 +2459,13 @@
     </row>
     <row r="54" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>11</v>
@@ -2281,13 +2485,13 @@
     </row>
     <row r="55" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>11</v>
@@ -2307,13 +2511,13 @@
     </row>
     <row r="56" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>11</v>
@@ -2333,13 +2537,13 @@
     </row>
     <row r="57" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>11</v>
@@ -2359,13 +2563,13 @@
     </row>
     <row r="58" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>11</v>
@@ -2385,13 +2589,13 @@
     </row>
     <row r="59" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>11</v>
@@ -2411,13 +2615,13 @@
     </row>
     <row r="60" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>11</v>
@@ -2437,13 +2641,13 @@
     </row>
     <row r="61" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>11</v>
@@ -2463,13 +2667,13 @@
     </row>
     <row r="62" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>11</v>
@@ -2489,13 +2693,13 @@
     </row>
     <row r="63" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>11</v>
@@ -2515,13 +2719,13 @@
     </row>
     <row r="64" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>11</v>
@@ -2541,13 +2745,13 @@
     </row>
     <row r="65" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>11</v>
@@ -2567,13 +2771,13 @@
     </row>
     <row r="66" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>11</v>
@@ -2593,13 +2797,13 @@
     </row>
     <row r="67" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>11</v>
@@ -2619,13 +2823,13 @@
     </row>
     <row r="68" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>11</v>
@@ -2645,13 +2849,13 @@
     </row>
     <row r="69" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>11</v>
@@ -2671,13 +2875,13 @@
     </row>
     <row r="70" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>11</v>
@@ -2697,13 +2901,13 @@
     </row>
     <row r="71" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>11</v>
@@ -2723,13 +2927,13 @@
     </row>
     <row r="72" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D72" s="2" t="s">
         <v>11</v>
@@ -2749,13 +2953,13 @@
     </row>
     <row r="73" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>11</v>
@@ -2775,13 +2979,13 @@
     </row>
     <row r="74" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D74" s="2" t="s">
         <v>11</v>
@@ -2801,13 +3005,13 @@
     </row>
     <row r="75" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D75" s="2" t="s">
         <v>11</v>
@@ -2827,13 +3031,13 @@
     </row>
     <row r="76" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D76" s="2" t="s">
         <v>11</v>
@@ -2853,13 +3057,13 @@
     </row>
     <row r="77" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D77" s="2" t="s">
         <v>11</v>
@@ -2879,13 +3083,13 @@
     </row>
     <row r="78" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D78" s="2" t="s">
         <v>11</v>
@@ -2905,13 +3109,13 @@
     </row>
     <row r="79" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D79" s="2" t="s">
         <v>11</v>
@@ -2931,13 +3135,13 @@
     </row>
     <row r="80" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D80" s="2" t="s">
         <v>11</v>
@@ -2957,13 +3161,13 @@
     </row>
     <row r="81" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D81" s="2" t="s">
         <v>11</v>
@@ -2983,13 +3187,13 @@
     </row>
     <row r="82" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D82" s="2" t="s">
         <v>11</v>
@@ -3009,22 +3213,22 @@
     </row>
     <row r="83" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>11</v>
+        <v>111</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>11</v>
+        <v>112</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G83" s="2" t="s">
         <v>11</v>
@@ -3035,22 +3239,22 @@
     </row>
     <row r="84" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>11</v>
+        <v>111</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>11</v>
+        <v>114</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G84" s="2" t="s">
         <v>11</v>
@@ -3061,22 +3265,22 @@
     </row>
     <row r="85" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>11</v>
+        <v>111</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>11</v>
+        <v>114</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G85" s="2" t="s">
         <v>11</v>
@@ -3087,22 +3291,22 @@
     </row>
     <row r="86" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>11</v>
+        <v>111</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>11</v>
+        <v>114</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G86" s="2" t="s">
         <v>11</v>
@@ -3113,22 +3317,22 @@
     </row>
     <row r="87" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>11</v>
+        <v>111</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>11</v>
+        <v>118</v>
       </c>
       <c r="F87" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G87" s="2" t="s">
         <v>11</v>
@@ -3139,22 +3343,22 @@
     </row>
     <row r="88" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>70</v>
+        <v>120</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="D88" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>11</v>
+        <v>112</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G88" s="2" t="s">
         <v>11</v>
@@ -3165,22 +3369,22 @@
     </row>
     <row r="89" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>70</v>
+        <v>120</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="D89" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>11</v>
+        <v>112</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G89" s="2" t="s">
         <v>11</v>
@@ -3191,22 +3395,22 @@
     </row>
     <row r="90" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>70</v>
+        <v>120</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="D90" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>11</v>
+        <v>112</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G90" s="2" t="s">
         <v>11</v>
@@ -3217,22 +3421,22 @@
     </row>
     <row r="91" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>70</v>
+        <v>120</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="D91" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>11</v>
+        <v>112</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G91" s="2" t="s">
         <v>11</v>
@@ -3243,13 +3447,13 @@
     </row>
     <row r="92" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>70</v>
+        <v>125</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="D92" s="2" t="s">
         <v>11</v>
@@ -3258,7 +3462,7 @@
         <v>11</v>
       </c>
       <c r="F92" s="2" t="s">
-        <v>11</v>
+        <v>126</v>
       </c>
       <c r="G92" s="2" t="s">
         <v>11</v>
@@ -3269,13 +3473,13 @@
     </row>
     <row r="93" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>70</v>
+        <v>125</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="D93" s="2" t="s">
         <v>11</v>
@@ -3284,7 +3488,7 @@
         <v>11</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>11</v>
+        <v>126</v>
       </c>
       <c r="G93" s="2" t="s">
         <v>11</v>
@@ -3295,13 +3499,13 @@
     </row>
     <row r="94" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>70</v>
+        <v>125</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="D94" s="2" t="s">
         <v>11</v>
@@ -3310,7 +3514,7 @@
         <v>11</v>
       </c>
       <c r="F94" s="2" t="s">
-        <v>11</v>
+        <v>126</v>
       </c>
       <c r="G94" s="2" t="s">
         <v>11</v>
@@ -3321,13 +3525,13 @@
     </row>
     <row r="95" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>70</v>
+        <v>125</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="D95" s="2" t="s">
         <v>11</v>
@@ -3336,7 +3540,7 @@
         <v>11</v>
       </c>
       <c r="F95" s="2" t="s">
-        <v>11</v>
+        <v>126</v>
       </c>
       <c r="G95" s="2" t="s">
         <v>11</v>
@@ -3347,22 +3551,22 @@
     </row>
     <row r="96" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>70</v>
+        <v>131</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>11</v>
+        <v>132</v>
       </c>
       <c r="E96" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F96" s="2" t="s">
-        <v>11</v>
+        <v>133</v>
       </c>
       <c r="G96" s="2" t="s">
         <v>11</v>
@@ -3373,22 +3577,22 @@
     </row>
     <row r="97" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>70</v>
+        <v>131</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>11</v>
+        <v>132</v>
       </c>
       <c r="E97" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F97" s="2" t="s">
-        <v>11</v>
+        <v>133</v>
       </c>
       <c r="G97" s="2" t="s">
         <v>11</v>
@@ -3399,22 +3603,22 @@
     </row>
     <row r="98" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>11</v>
+        <v>132</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>138</v>
+        <v>11</v>
       </c>
       <c r="F98" s="2" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="G98" s="2" t="s">
         <v>11</v>
@@ -3425,22 +3629,22 @@
     </row>
     <row r="99" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>142</v>
+        <v>11</v>
       </c>
       <c r="F99" s="2" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="G99" s="2" t="s">
         <v>11</v>
@@ -3451,22 +3655,22 @@
     </row>
     <row r="100" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>63</v>
+        <v>139</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>144</v>
+        <v>11</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>145</v>
+        <v>11</v>
       </c>
       <c r="F100" s="2" t="s">
-        <v>139</v>
+        <v>11</v>
       </c>
       <c r="G100" s="2" t="s">
         <v>11</v>
@@ -3477,32 +3681,1774 @@
     </row>
     <row r="101" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E101" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F101" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G101" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H101" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E102" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F102" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G102" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H102" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A103" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B103" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E103" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F103" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G103" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H103" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E104" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F104" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G104" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H104" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A105" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E105" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F105" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G105" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H105" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A106" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E106" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F106" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G106" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H106" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A107" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="B101" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="C101" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D101" s="2" t="s">
+      <c r="B107" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E107" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F107" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G107" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H107" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A108" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="E101" s="2" t="s">
+      <c r="B108" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E108" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F108" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G108" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H108" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A109" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="F101" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G101" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H101" s="4" t="s">
+      <c r="B109" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D109" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E109" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F109" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G109" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H109" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A110" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="B110" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D110" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E110" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F110" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G110" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H110" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A111" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="B111" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C111" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D111" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E111" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F111" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G111" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H111" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A112" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="B112" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C112" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D112" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E112" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F112" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G112" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H112" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="113" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A113" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="B113" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C113" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D113" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E113" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F113" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G113" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H113" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A114" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="B114" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D114" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E114" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F114" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G114" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H114" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A115" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B115" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D115" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E115" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F115" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G115" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H115" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A116" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="B116" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D116" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E116" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F116" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G116" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H116" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="117" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A117" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="B117" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C117" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E117" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F117" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G117" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H117" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="118" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A118" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="B118" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C118" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D118" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E118" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F118" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G118" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H118" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="119" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A119" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="B119" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C119" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E119" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F119" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G119" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H119" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="120" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A120" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B120" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D120" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E120" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F120" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G120" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H120" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="121" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A121" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="B121" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C121" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D121" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E121" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F121" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G121" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H121" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A122" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="B122" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C122" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D122" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E122" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F122" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G122" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H122" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="123" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A123" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="B123" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C123" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D123" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E123" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F123" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G123" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H123" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="124" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A124" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B124" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E124" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F124" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G124" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H124" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="125" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A125" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B125" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C125" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D125" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E125" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F125" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G125" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H125" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="126" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A126" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B126" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C126" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D126" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E126" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F126" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G126" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H126" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A127" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="B127" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D127" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E127" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F127" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G127" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H127" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="128" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A128" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="B128" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C128" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D128" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E128" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F128" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G128" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H128" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="129" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A129" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="B129" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C129" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D129" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E129" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F129" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G129" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H129" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="130" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A130" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="B130" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C130" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D130" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E130" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F130" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G130" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H130" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="131" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A131" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="B131" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C131" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D131" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E131" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F131" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G131" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H131" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="132" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A132" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D132" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E132" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F132" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G132" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H132" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="133" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A133" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="B133" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D133" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E133" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F133" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G133" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H133" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="134" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A134" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="B134" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C134" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D134" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E134" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F134" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G134" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H134" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="135" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A135" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="B135" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D135" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E135" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F135" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G135" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H135" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="136" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A136" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="B136" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C136" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D136" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E136" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F136" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G136" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H136" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="137" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A137" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="B137" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C137" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D137" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E137" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F137" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G137" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H137" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="138" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A138" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="B138" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C138" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D138" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E138" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F138" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G138" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H138" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="139" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A139" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="B139" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C139" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D139" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E139" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F139" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G139" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H139" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="140" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A140" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="B140" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C140" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D140" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E140" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F140" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G140" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H140" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="141" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A141" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="B141" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C141" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D141" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E141" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F141" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G141" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H141" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="142" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A142" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B142" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C142" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D142" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E142" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F142" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G142" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H142" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="143" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A143" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="B143" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C143" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D143" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E143" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F143" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G143" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H143" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="144" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A144" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="B144" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C144" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D144" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E144" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F144" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G144" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H144" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="145" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A145" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="B145" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C145" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D145" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E145" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F145" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G145" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H145" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="146" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A146" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D146" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E146" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F146" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G146" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H146" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="147" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A147" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="B147" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C147" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D147" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E147" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F147" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G147" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H147" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="148" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A148" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="B148" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C148" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D148" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E148" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F148" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G148" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H148" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="149" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A149" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="B149" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C149" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D149" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E149" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F149" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G149" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H149" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="150" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A150" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B150" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C150" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D150" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E150" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F150" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G150" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H150" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="151" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A151" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="B151" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C151" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D151" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E151" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F151" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G151" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H151" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="152" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A152" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="B152" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D152" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E152" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F152" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G152" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H152" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="153" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A153" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="B153" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C153" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D153" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E153" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F153" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G153" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H153" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="154" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A154" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B154" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C154" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D154" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E154" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F154" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G154" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H154" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="155" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A155" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B155" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C155" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D155" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E155" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F155" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G155" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H155" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="156" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A156" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="B156" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C156" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D156" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E156" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F156" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G156" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H156" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="157" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A157" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="B157" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C157" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D157" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E157" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F157" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G157" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H157" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="158" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A158" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="B158" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C158" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D158" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E158" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F158" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G158" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H158" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="159" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A159" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="B159" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C159" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D159" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E159" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F159" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G159" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H159" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="160" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A160" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="B160" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C160" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D160" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E160" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F160" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G160" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H160" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="161" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A161" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="B161" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C161" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D161" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E161" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F161" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G161" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H161" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="162" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A162" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="B162" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C162" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D162" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E162" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F162" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G162" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H162" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="163" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A163" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="B163" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C163" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D163" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E163" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F163" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G163" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H163" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="164" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A164" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="B164" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C164" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D164" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E164" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F164" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G164" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H164" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="165" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A165" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="B165" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="C165" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D165" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E165" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="F165" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="G165" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H165" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="166" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A166" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="B166" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="C166" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D166" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="E166" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="F166" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="G166" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H166" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="167" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A167" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="B167" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="C167" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D167" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="E167" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="F167" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="G167" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H167" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="168" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A168" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="B168" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="C168" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D168" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E168" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="F168" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="G168" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H168" s="4" t="s">
         <v>14</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H101"/>
+  <autoFilter ref="A1:H168"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Renumber the collection so the references read in order
M. D. Ishak's paintings sat at IAC-101 onward while hanging after
IAC-014, which read as erratic. The whole collection is renumbered in
hanging order: Ishak is now IAC-015 to IAC-081 and the painters after
him shift up to IAC-082 to IAC-167.

Renumbering is a deliberate act, so it lives behind a flag rather than
happening on every build:

    node scripts/build-catalog.cjs --renumber

Fixed alongside it: spreadsheet rows are keyed by reference, so after a
renumber every row's title and size would have landed on whichever
painting inherited its old number. `asRef` now translates a row's
reference back through the previous refs.json to the photograph it means
before matching. Verified afterwards that all 167 works still carry the
title and size recorded for their own photograph.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Uv8R3RW9M9MhGG8c2qV64h
</commit_message>
<xml_diff>
--- a/Indus Art Collection - Catalogue.xlsx
+++ b/Indus Art Collection - Catalogue.xlsx
@@ -133,15 +133,312 @@
     <t>153 x 191 cm</t>
   </si>
   <si>
+    <t>IAC-015</t>
+  </si>
+  <si>
+    <t>M. D. Ishak</t>
+  </si>
+  <si>
+    <t>Traditional</t>
+  </si>
+  <si>
+    <t>IAC-016</t>
+  </si>
+  <si>
+    <t>IAC-017</t>
+  </si>
+  <si>
+    <t>IAC-018</t>
+  </si>
+  <si>
+    <t>IAC-019</t>
+  </si>
+  <si>
+    <t>IAC-020</t>
+  </si>
+  <si>
+    <t>IAC-021</t>
+  </si>
+  <si>
+    <t>IAC-022</t>
+  </si>
+  <si>
+    <t>IAC-023</t>
+  </si>
+  <si>
+    <t>IAC-024</t>
+  </si>
+  <si>
+    <t>IAC-025</t>
+  </si>
+  <si>
+    <t>IAC-026</t>
+  </si>
+  <si>
+    <t>IAC-027</t>
+  </si>
+  <si>
+    <t>IAC-028</t>
+  </si>
+  <si>
+    <t>IAC-029</t>
+  </si>
+  <si>
+    <t>IAC-030</t>
+  </si>
+  <si>
+    <t>IAC-031</t>
+  </si>
+  <si>
+    <t>IAC-032</t>
+  </si>
+  <si>
+    <t>IAC-033</t>
+  </si>
+  <si>
+    <t>IAC-034</t>
+  </si>
+  <si>
+    <t>IAC-035</t>
+  </si>
+  <si>
+    <t>IAC-036</t>
+  </si>
+  <si>
+    <t>IAC-037</t>
+  </si>
+  <si>
+    <t>IAC-038</t>
+  </si>
+  <si>
+    <t>IAC-039</t>
+  </si>
+  <si>
+    <t>IAC-040</t>
+  </si>
+  <si>
+    <t>IAC-041</t>
+  </si>
+  <si>
+    <t>IAC-042</t>
+  </si>
+  <si>
+    <t>IAC-043</t>
+  </si>
+  <si>
+    <t>IAC-044</t>
+  </si>
+  <si>
+    <t>IAC-045</t>
+  </si>
+  <si>
+    <t>IAC-046</t>
+  </si>
+  <si>
+    <t>IAC-047</t>
+  </si>
+  <si>
+    <t>IAC-048</t>
+  </si>
+  <si>
+    <t>IAC-049</t>
+  </si>
+  <si>
+    <t>IAC-050</t>
+  </si>
+  <si>
+    <t>IAC-051</t>
+  </si>
+  <si>
+    <t>IAC-052</t>
+  </si>
+  <si>
+    <t>IAC-053</t>
+  </si>
+  <si>
+    <t>IAC-054</t>
+  </si>
+  <si>
+    <t>IAC-055</t>
+  </si>
+  <si>
+    <t>IAC-056</t>
+  </si>
+  <si>
+    <t>IAC-057</t>
+  </si>
+  <si>
+    <t>IAC-058</t>
+  </si>
+  <si>
+    <t>IAC-059</t>
+  </si>
+  <si>
+    <t>IAC-060</t>
+  </si>
+  <si>
+    <t>IAC-061</t>
+  </si>
+  <si>
+    <t>IAC-062</t>
+  </si>
+  <si>
+    <t>IAC-063</t>
+  </si>
+  <si>
+    <t>IAC-064</t>
+  </si>
+  <si>
+    <t>IAC-065</t>
+  </si>
+  <si>
+    <t>IAC-066</t>
+  </si>
+  <si>
+    <t>IAC-067</t>
+  </si>
+  <si>
+    <t>IAC-068</t>
+  </si>
+  <si>
+    <t>IAC-069</t>
+  </si>
+  <si>
+    <t>IAC-070</t>
+  </si>
+  <si>
+    <t>IAC-071</t>
+  </si>
+  <si>
+    <t>IAC-072</t>
+  </si>
+  <si>
+    <t>IAC-073</t>
+  </si>
+  <si>
+    <t>IAC-074</t>
+  </si>
+  <si>
+    <t>IAC-075</t>
+  </si>
+  <si>
+    <t>IAC-076</t>
+  </si>
+  <si>
+    <t>IAC-077</t>
+  </si>
+  <si>
+    <t>IAC-078</t>
+  </si>
+  <si>
+    <t>IAC-079</t>
+  </si>
+  <si>
+    <t>IAC-080</t>
+  </si>
+  <si>
+    <t>IAC-081</t>
+  </si>
+  <si>
+    <t>IAC-082</t>
+  </si>
+  <si>
+    <t>Ashok Rathod</t>
+  </si>
+  <si>
+    <t>Nandi</t>
+  </si>
+  <si>
+    <t>24 x 24 in</t>
+  </si>
+  <si>
+    <t>IAC-083</t>
+  </si>
+  <si>
+    <t>36 x 60 in</t>
+  </si>
+  <si>
+    <t>IAC-084</t>
+  </si>
+  <si>
+    <t>IAC-085</t>
+  </si>
+  <si>
+    <t>IAC-086</t>
+  </si>
+  <si>
+    <t>48 x 72 in</t>
+  </si>
+  <si>
+    <t>IAC-087</t>
+  </si>
+  <si>
+    <t>Gopal Naskar</t>
+  </si>
+  <si>
+    <t>IAC-088</t>
+  </si>
+  <si>
+    <t>IAC-089</t>
+  </si>
+  <si>
+    <t>IAC-090</t>
+  </si>
+  <si>
+    <t>IAC-091</t>
+  </si>
+  <si>
+    <t>Umendra P. Singh</t>
+  </si>
+  <si>
+    <t>Oil on Canvas</t>
+  </si>
+  <si>
+    <t>IAC-092</t>
+  </si>
+  <si>
+    <t>IAC-093</t>
+  </si>
+  <si>
+    <t>IAC-094</t>
+  </si>
+  <si>
+    <t>IAC-095</t>
+  </si>
+  <si>
+    <t>M. Salim</t>
+  </si>
+  <si>
+    <t>Landscape</t>
+  </si>
+  <si>
+    <t>Mix Medium</t>
+  </si>
+  <si>
+    <t>IAC-096</t>
+  </si>
+  <si>
+    <t>IAC-097</t>
+  </si>
+  <si>
+    <t>IAC-098</t>
+  </si>
+  <si>
+    <t>IAC-099</t>
+  </si>
+  <si>
+    <t>Folk &amp; Tribal Masters</t>
+  </si>
+  <si>
+    <t>Folk</t>
+  </si>
+  <si>
+    <t>IAC-100</t>
+  </si>
+  <si>
     <t>IAC-101</t>
   </si>
   <si>
-    <t>M. D. Ishak</t>
-  </si>
-  <si>
-    <t>Traditional</t>
-  </si>
-  <si>
     <t>IAC-102</t>
   </si>
   <si>
@@ -331,331 +628,34 @@
     <t>IAC-164</t>
   </si>
   <si>
+    <t>N. K. Mishra</t>
+  </si>
+  <si>
+    <t>21.5 x 15 in</t>
+  </si>
+  <si>
+    <t>Water colour and gouache on paper</t>
+  </si>
+  <si>
     <t>IAC-165</t>
   </si>
   <si>
+    <t>Parvati and Ganesha</t>
+  </si>
+  <si>
+    <t>13.2 x 7.1 in</t>
+  </si>
+  <si>
     <t>IAC-166</t>
   </si>
   <si>
+    <t>Ganesh</t>
+  </si>
+  <si>
+    <t>12.5 x 8.5 in</t>
+  </si>
+  <si>
     <t>IAC-167</t>
-  </si>
-  <si>
-    <t>IAC-015</t>
-  </si>
-  <si>
-    <t>Ashok Rathod</t>
-  </si>
-  <si>
-    <t>Nandi</t>
-  </si>
-  <si>
-    <t>24 x 24 in</t>
-  </si>
-  <si>
-    <t>IAC-016</t>
-  </si>
-  <si>
-    <t>36 x 60 in</t>
-  </si>
-  <si>
-    <t>IAC-017</t>
-  </si>
-  <si>
-    <t>IAC-018</t>
-  </si>
-  <si>
-    <t>IAC-019</t>
-  </si>
-  <si>
-    <t>48 x 72 in</t>
-  </si>
-  <si>
-    <t>IAC-020</t>
-  </si>
-  <si>
-    <t>Gopal Naskar</t>
-  </si>
-  <si>
-    <t>IAC-021</t>
-  </si>
-  <si>
-    <t>IAC-022</t>
-  </si>
-  <si>
-    <t>IAC-023</t>
-  </si>
-  <si>
-    <t>IAC-024</t>
-  </si>
-  <si>
-    <t>Umendra P. Singh</t>
-  </si>
-  <si>
-    <t>Oil on Canvas</t>
-  </si>
-  <si>
-    <t>IAC-025</t>
-  </si>
-  <si>
-    <t>IAC-026</t>
-  </si>
-  <si>
-    <t>IAC-027</t>
-  </si>
-  <si>
-    <t>IAC-028</t>
-  </si>
-  <si>
-    <t>M. Salim</t>
-  </si>
-  <si>
-    <t>Landscape</t>
-  </si>
-  <si>
-    <t>Mix Medium</t>
-  </si>
-  <si>
-    <t>IAC-029</t>
-  </si>
-  <si>
-    <t>IAC-030</t>
-  </si>
-  <si>
-    <t>IAC-031</t>
-  </si>
-  <si>
-    <t>IAC-032</t>
-  </si>
-  <si>
-    <t>Folk &amp; Tribal Masters</t>
-  </si>
-  <si>
-    <t>Folk</t>
-  </si>
-  <si>
-    <t>IAC-033</t>
-  </si>
-  <si>
-    <t>IAC-034</t>
-  </si>
-  <si>
-    <t>IAC-035</t>
-  </si>
-  <si>
-    <t>IAC-036</t>
-  </si>
-  <si>
-    <t>IAC-037</t>
-  </si>
-  <si>
-    <t>IAC-038</t>
-  </si>
-  <si>
-    <t>IAC-039</t>
-  </si>
-  <si>
-    <t>IAC-040</t>
-  </si>
-  <si>
-    <t>IAC-041</t>
-  </si>
-  <si>
-    <t>IAC-042</t>
-  </si>
-  <si>
-    <t>IAC-043</t>
-  </si>
-  <si>
-    <t>IAC-044</t>
-  </si>
-  <si>
-    <t>IAC-045</t>
-  </si>
-  <si>
-    <t>IAC-046</t>
-  </si>
-  <si>
-    <t>IAC-047</t>
-  </si>
-  <si>
-    <t>IAC-048</t>
-  </si>
-  <si>
-    <t>IAC-049</t>
-  </si>
-  <si>
-    <t>IAC-050</t>
-  </si>
-  <si>
-    <t>IAC-051</t>
-  </si>
-  <si>
-    <t>IAC-052</t>
-  </si>
-  <si>
-    <t>IAC-053</t>
-  </si>
-  <si>
-    <t>IAC-054</t>
-  </si>
-  <si>
-    <t>IAC-055</t>
-  </si>
-  <si>
-    <t>IAC-056</t>
-  </si>
-  <si>
-    <t>IAC-057</t>
-  </si>
-  <si>
-    <t>IAC-058</t>
-  </si>
-  <si>
-    <t>IAC-059</t>
-  </si>
-  <si>
-    <t>IAC-060</t>
-  </si>
-  <si>
-    <t>IAC-061</t>
-  </si>
-  <si>
-    <t>IAC-062</t>
-  </si>
-  <si>
-    <t>IAC-063</t>
-  </si>
-  <si>
-    <t>IAC-064</t>
-  </si>
-  <si>
-    <t>IAC-065</t>
-  </si>
-  <si>
-    <t>IAC-066</t>
-  </si>
-  <si>
-    <t>IAC-067</t>
-  </si>
-  <si>
-    <t>IAC-068</t>
-  </si>
-  <si>
-    <t>IAC-069</t>
-  </si>
-  <si>
-    <t>IAC-070</t>
-  </si>
-  <si>
-    <t>IAC-071</t>
-  </si>
-  <si>
-    <t>IAC-072</t>
-  </si>
-  <si>
-    <t>IAC-073</t>
-  </si>
-  <si>
-    <t>IAC-074</t>
-  </si>
-  <si>
-    <t>IAC-075</t>
-  </si>
-  <si>
-    <t>IAC-076</t>
-  </si>
-  <si>
-    <t>IAC-077</t>
-  </si>
-  <si>
-    <t>IAC-078</t>
-  </si>
-  <si>
-    <t>IAC-079</t>
-  </si>
-  <si>
-    <t>IAC-080</t>
-  </si>
-  <si>
-    <t>IAC-081</t>
-  </si>
-  <si>
-    <t>IAC-082</t>
-  </si>
-  <si>
-    <t>IAC-083</t>
-  </si>
-  <si>
-    <t>IAC-084</t>
-  </si>
-  <si>
-    <t>IAC-085</t>
-  </si>
-  <si>
-    <t>IAC-086</t>
-  </si>
-  <si>
-    <t>IAC-087</t>
-  </si>
-  <si>
-    <t>IAC-088</t>
-  </si>
-  <si>
-    <t>IAC-089</t>
-  </si>
-  <si>
-    <t>IAC-090</t>
-  </si>
-  <si>
-    <t>IAC-091</t>
-  </si>
-  <si>
-    <t>IAC-092</t>
-  </si>
-  <si>
-    <t>IAC-093</t>
-  </si>
-  <si>
-    <t>IAC-094</t>
-  </si>
-  <si>
-    <t>IAC-095</t>
-  </si>
-  <si>
-    <t>IAC-096</t>
-  </si>
-  <si>
-    <t>IAC-097</t>
-  </si>
-  <si>
-    <t>N. K. Mishra</t>
-  </si>
-  <si>
-    <t>21.5 x 15 in</t>
-  </si>
-  <si>
-    <t>Water colour and gouache on paper</t>
-  </si>
-  <si>
-    <t>IAC-098</t>
-  </si>
-  <si>
-    <t>Parvati and Ganesha</t>
-  </si>
-  <si>
-    <t>13.2 x 7.1 in</t>
-  </si>
-  <si>
-    <t>IAC-099</t>
-  </si>
-  <si>
-    <t>Ganesh</t>
-  </si>
-  <si>
-    <t>12.5 x 8.5 in</t>
-  </si>
-  <si>
-    <t>IAC-100</t>
   </si>
   <si>
     <t>Hanuman</t>

</xml_diff>

<commit_message>
Replace the featured section with a rotating New Collection
The home page was showing a dozen paintings the gallery already holds,
which read as repetition. That section is now "New Collection": a
selection chosen by reference number in NEW_COLLECTION in config.ts —
this week Umesh Kumar Saxena (IAC-001 to IAC-008) and Kandan G (IAC-009
to IAC-012) — meant to be changed weekly. A mistyped reference is
skipped, and if none match the first twelve works stand in so the page
is never bare.

The gallery's tabs are now Modern, Contemporary, Abstract,
Impressionism, Realism and Traditional Folk Art, ordered by STYLE_ORDER
in config.ts and rendered only when the collection holds work of that
kind — so a style can be listed before its first painting arrives.
Each painter's category is the `style` line in metadata.cjs.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Uv8R3RW9M9MhGG8c2qV64h
</commit_message>
<xml_diff>
--- a/Indus Art Collection - Catalogue.xlsx
+++ b/Indus Art Collection - Catalogue.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1344" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1344" uniqueCount="220">
   <si>
     <t>Reference (do not edit)</t>
   </si>
@@ -43,309 +43,315 @@
     <t>Umesh Kumar Saxena</t>
   </si>
   <si>
+    <t>Abstract</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>70 x 70 in / 178 x 178 cm</t>
+  </si>
+  <si>
+    <t>Acrylic on canvas</t>
+  </si>
+  <si>
+    <t>Add a short description of this painting here.</t>
+  </si>
+  <si>
+    <t>IAC-002</t>
+  </si>
+  <si>
+    <t>36 x 72 in</t>
+  </si>
+  <si>
+    <t>2025</t>
+  </si>
+  <si>
+    <t>IAC-003</t>
+  </si>
+  <si>
+    <t>IAC-004</t>
+  </si>
+  <si>
+    <t>IAC-005</t>
+  </si>
+  <si>
+    <t>IAC-006</t>
+  </si>
+  <si>
+    <t>IAC-007</t>
+  </si>
+  <si>
+    <t>Triptych</t>
+  </si>
+  <si>
+    <t>18 x 60 in each</t>
+  </si>
+  <si>
+    <t>IAC-008</t>
+  </si>
+  <si>
+    <t>IAC-009</t>
+  </si>
+  <si>
+    <t>Kandan G</t>
+  </si>
+  <si>
+    <t>Modern</t>
+  </si>
+  <si>
+    <t>Banaras Series</t>
+  </si>
+  <si>
+    <t>24 x 48 in / 61 x 122 cm</t>
+  </si>
+  <si>
+    <t>2024</t>
+  </si>
+  <si>
+    <t>IAC-010</t>
+  </si>
+  <si>
+    <t>IAC-011</t>
+  </si>
+  <si>
+    <t>36 x 60 in / 92 x 153 cm</t>
+  </si>
+  <si>
+    <t>IAC-012</t>
+  </si>
+  <si>
+    <t>IAC-013</t>
+  </si>
+  <si>
+    <t>Nirakar Chowdhury</t>
+  </si>
+  <si>
+    <t>140 x 85 cm</t>
+  </si>
+  <si>
+    <t>IAC-014</t>
+  </si>
+  <si>
+    <t>153 x 191 cm</t>
+  </si>
+  <si>
+    <t>IAC-015</t>
+  </si>
+  <si>
+    <t>M. D. Ishak</t>
+  </si>
+  <si>
+    <t>Realism</t>
+  </si>
+  <si>
+    <t>IAC-016</t>
+  </si>
+  <si>
+    <t>IAC-017</t>
+  </si>
+  <si>
+    <t>IAC-018</t>
+  </si>
+  <si>
+    <t>IAC-019</t>
+  </si>
+  <si>
+    <t>IAC-020</t>
+  </si>
+  <si>
+    <t>IAC-021</t>
+  </si>
+  <si>
+    <t>IAC-022</t>
+  </si>
+  <si>
+    <t>IAC-023</t>
+  </si>
+  <si>
+    <t>IAC-024</t>
+  </si>
+  <si>
+    <t>IAC-025</t>
+  </si>
+  <si>
+    <t>IAC-026</t>
+  </si>
+  <si>
+    <t>IAC-027</t>
+  </si>
+  <si>
+    <t>IAC-028</t>
+  </si>
+  <si>
+    <t>IAC-029</t>
+  </si>
+  <si>
+    <t>IAC-030</t>
+  </si>
+  <si>
+    <t>IAC-031</t>
+  </si>
+  <si>
+    <t>IAC-032</t>
+  </si>
+  <si>
+    <t>IAC-033</t>
+  </si>
+  <si>
+    <t>IAC-034</t>
+  </si>
+  <si>
+    <t>IAC-035</t>
+  </si>
+  <si>
+    <t>IAC-036</t>
+  </si>
+  <si>
+    <t>IAC-037</t>
+  </si>
+  <si>
+    <t>IAC-038</t>
+  </si>
+  <si>
+    <t>IAC-039</t>
+  </si>
+  <si>
+    <t>IAC-040</t>
+  </si>
+  <si>
+    <t>IAC-041</t>
+  </si>
+  <si>
+    <t>IAC-042</t>
+  </si>
+  <si>
+    <t>IAC-043</t>
+  </si>
+  <si>
+    <t>IAC-044</t>
+  </si>
+  <si>
+    <t>IAC-045</t>
+  </si>
+  <si>
+    <t>IAC-046</t>
+  </si>
+  <si>
+    <t>IAC-047</t>
+  </si>
+  <si>
+    <t>IAC-048</t>
+  </si>
+  <si>
+    <t>IAC-049</t>
+  </si>
+  <si>
+    <t>IAC-050</t>
+  </si>
+  <si>
+    <t>IAC-051</t>
+  </si>
+  <si>
+    <t>IAC-052</t>
+  </si>
+  <si>
+    <t>IAC-053</t>
+  </si>
+  <si>
+    <t>IAC-054</t>
+  </si>
+  <si>
+    <t>IAC-055</t>
+  </si>
+  <si>
+    <t>IAC-056</t>
+  </si>
+  <si>
+    <t>IAC-057</t>
+  </si>
+  <si>
+    <t>IAC-058</t>
+  </si>
+  <si>
+    <t>IAC-059</t>
+  </si>
+  <si>
+    <t>IAC-060</t>
+  </si>
+  <si>
+    <t>IAC-061</t>
+  </si>
+  <si>
+    <t>IAC-062</t>
+  </si>
+  <si>
+    <t>IAC-063</t>
+  </si>
+  <si>
+    <t>IAC-064</t>
+  </si>
+  <si>
+    <t>IAC-065</t>
+  </si>
+  <si>
+    <t>IAC-066</t>
+  </si>
+  <si>
+    <t>IAC-067</t>
+  </si>
+  <si>
+    <t>IAC-068</t>
+  </si>
+  <si>
+    <t>IAC-069</t>
+  </si>
+  <si>
+    <t>IAC-070</t>
+  </si>
+  <si>
+    <t>IAC-071</t>
+  </si>
+  <si>
+    <t>IAC-072</t>
+  </si>
+  <si>
+    <t>IAC-073</t>
+  </si>
+  <si>
+    <t>IAC-074</t>
+  </si>
+  <si>
+    <t>IAC-075</t>
+  </si>
+  <si>
+    <t>IAC-076</t>
+  </si>
+  <si>
+    <t>IAC-077</t>
+  </si>
+  <si>
+    <t>IAC-078</t>
+  </si>
+  <si>
+    <t>IAC-079</t>
+  </si>
+  <si>
+    <t>IAC-080</t>
+  </si>
+  <si>
+    <t>IAC-081</t>
+  </si>
+  <si>
+    <t>IAC-082</t>
+  </si>
+  <si>
+    <t>Ashok Rathod</t>
+  </si>
+  <si>
     <t>Contemporary</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>70 x 70 in / 178 x 178 cm</t>
-  </si>
-  <si>
-    <t>Acrylic on canvas</t>
-  </si>
-  <si>
-    <t>Add a short description of this painting here.</t>
-  </si>
-  <si>
-    <t>IAC-002</t>
-  </si>
-  <si>
-    <t>36 x 72 in</t>
-  </si>
-  <si>
-    <t>2025</t>
-  </si>
-  <si>
-    <t>IAC-003</t>
-  </si>
-  <si>
-    <t>IAC-004</t>
-  </si>
-  <si>
-    <t>IAC-005</t>
-  </si>
-  <si>
-    <t>IAC-006</t>
-  </si>
-  <si>
-    <t>IAC-007</t>
-  </si>
-  <si>
-    <t>Triptych</t>
-  </si>
-  <si>
-    <t>18 x 60 in each</t>
-  </si>
-  <si>
-    <t>IAC-008</t>
-  </si>
-  <si>
-    <t>IAC-009</t>
-  </si>
-  <si>
-    <t>Kandan G</t>
-  </si>
-  <si>
-    <t>Banaras Series</t>
-  </si>
-  <si>
-    <t>24 x 48 in / 61 x 122 cm</t>
-  </si>
-  <si>
-    <t>2024</t>
-  </si>
-  <si>
-    <t>IAC-010</t>
-  </si>
-  <si>
-    <t>IAC-011</t>
-  </si>
-  <si>
-    <t>36 x 60 in / 92 x 153 cm</t>
-  </si>
-  <si>
-    <t>IAC-012</t>
-  </si>
-  <si>
-    <t>IAC-013</t>
-  </si>
-  <si>
-    <t>Nirakar Chowdhury</t>
-  </si>
-  <si>
-    <t>140 x 85 cm</t>
-  </si>
-  <si>
-    <t>IAC-014</t>
-  </si>
-  <si>
-    <t>153 x 191 cm</t>
-  </si>
-  <si>
-    <t>IAC-015</t>
-  </si>
-  <si>
-    <t>M. D. Ishak</t>
-  </si>
-  <si>
-    <t>Traditional</t>
-  </si>
-  <si>
-    <t>IAC-016</t>
-  </si>
-  <si>
-    <t>IAC-017</t>
-  </si>
-  <si>
-    <t>IAC-018</t>
-  </si>
-  <si>
-    <t>IAC-019</t>
-  </si>
-  <si>
-    <t>IAC-020</t>
-  </si>
-  <si>
-    <t>IAC-021</t>
-  </si>
-  <si>
-    <t>IAC-022</t>
-  </si>
-  <si>
-    <t>IAC-023</t>
-  </si>
-  <si>
-    <t>IAC-024</t>
-  </si>
-  <si>
-    <t>IAC-025</t>
-  </si>
-  <si>
-    <t>IAC-026</t>
-  </si>
-  <si>
-    <t>IAC-027</t>
-  </si>
-  <si>
-    <t>IAC-028</t>
-  </si>
-  <si>
-    <t>IAC-029</t>
-  </si>
-  <si>
-    <t>IAC-030</t>
-  </si>
-  <si>
-    <t>IAC-031</t>
-  </si>
-  <si>
-    <t>IAC-032</t>
-  </si>
-  <si>
-    <t>IAC-033</t>
-  </si>
-  <si>
-    <t>IAC-034</t>
-  </si>
-  <si>
-    <t>IAC-035</t>
-  </si>
-  <si>
-    <t>IAC-036</t>
-  </si>
-  <si>
-    <t>IAC-037</t>
-  </si>
-  <si>
-    <t>IAC-038</t>
-  </si>
-  <si>
-    <t>IAC-039</t>
-  </si>
-  <si>
-    <t>IAC-040</t>
-  </si>
-  <si>
-    <t>IAC-041</t>
-  </si>
-  <si>
-    <t>IAC-042</t>
-  </si>
-  <si>
-    <t>IAC-043</t>
-  </si>
-  <si>
-    <t>IAC-044</t>
-  </si>
-  <si>
-    <t>IAC-045</t>
-  </si>
-  <si>
-    <t>IAC-046</t>
-  </si>
-  <si>
-    <t>IAC-047</t>
-  </si>
-  <si>
-    <t>IAC-048</t>
-  </si>
-  <si>
-    <t>IAC-049</t>
-  </si>
-  <si>
-    <t>IAC-050</t>
-  </si>
-  <si>
-    <t>IAC-051</t>
-  </si>
-  <si>
-    <t>IAC-052</t>
-  </si>
-  <si>
-    <t>IAC-053</t>
-  </si>
-  <si>
-    <t>IAC-054</t>
-  </si>
-  <si>
-    <t>IAC-055</t>
-  </si>
-  <si>
-    <t>IAC-056</t>
-  </si>
-  <si>
-    <t>IAC-057</t>
-  </si>
-  <si>
-    <t>IAC-058</t>
-  </si>
-  <si>
-    <t>IAC-059</t>
-  </si>
-  <si>
-    <t>IAC-060</t>
-  </si>
-  <si>
-    <t>IAC-061</t>
-  </si>
-  <si>
-    <t>IAC-062</t>
-  </si>
-  <si>
-    <t>IAC-063</t>
-  </si>
-  <si>
-    <t>IAC-064</t>
-  </si>
-  <si>
-    <t>IAC-065</t>
-  </si>
-  <si>
-    <t>IAC-066</t>
-  </si>
-  <si>
-    <t>IAC-067</t>
-  </si>
-  <si>
-    <t>IAC-068</t>
-  </si>
-  <si>
-    <t>IAC-069</t>
-  </si>
-  <si>
-    <t>IAC-070</t>
-  </si>
-  <si>
-    <t>IAC-071</t>
-  </si>
-  <si>
-    <t>IAC-072</t>
-  </si>
-  <si>
-    <t>IAC-073</t>
-  </si>
-  <si>
-    <t>IAC-074</t>
-  </si>
-  <si>
-    <t>IAC-075</t>
-  </si>
-  <si>
-    <t>IAC-076</t>
-  </si>
-  <si>
-    <t>IAC-077</t>
-  </si>
-  <si>
-    <t>IAC-078</t>
-  </si>
-  <si>
-    <t>IAC-079</t>
-  </si>
-  <si>
-    <t>IAC-080</t>
-  </si>
-  <si>
-    <t>IAC-081</t>
-  </si>
-  <si>
-    <t>IAC-082</t>
-  </si>
-  <si>
-    <t>Ashok Rathod</t>
-  </si>
-  <si>
     <t>Nandi</t>
   </si>
   <si>
@@ -409,6 +415,9 @@
     <t>M. Salim</t>
   </si>
   <si>
+    <t>Impressionism</t>
+  </si>
+  <si>
     <t>Landscape</t>
   </si>
   <si>
@@ -430,7 +439,7 @@
     <t>Folk &amp; Tribal Masters</t>
   </si>
   <si>
-    <t>Folk</t>
+    <t>Traditional Folk Art</t>
   </si>
   <si>
     <t>IAC-100</t>
@@ -1321,19 +1330,19 @@
         <v>27</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>14</v>
@@ -1341,25 +1350,25 @@
     </row>
     <row r="11" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>27</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>14</v>
@@ -1367,19 +1376,19 @@
     </row>
     <row r="12" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>27</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>13</v>
@@ -1393,19 +1402,19 @@
     </row>
     <row r="13" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>27</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>13</v>
@@ -1419,19 +1428,19 @@
     </row>
     <row r="14" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>13</v>
@@ -1445,19 +1454,19 @@
     </row>
     <row r="15" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>13</v>
@@ -1471,13 +1480,13 @@
     </row>
     <row r="16" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>11</v>
@@ -1497,13 +1506,13 @@
     </row>
     <row r="17" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>11</v>
@@ -1523,13 +1532,13 @@
     </row>
     <row r="18" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>11</v>
@@ -1549,13 +1558,13 @@
     </row>
     <row r="19" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>11</v>
@@ -1575,13 +1584,13 @@
     </row>
     <row r="20" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>11</v>
@@ -1601,13 +1610,13 @@
     </row>
     <row r="21" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>11</v>
@@ -1627,13 +1636,13 @@
     </row>
     <row r="22" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>11</v>
@@ -1653,13 +1662,13 @@
     </row>
     <row r="23" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>11</v>
@@ -1679,13 +1688,13 @@
     </row>
     <row r="24" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>11</v>
@@ -1705,13 +1714,13 @@
     </row>
     <row r="25" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>11</v>
@@ -1731,13 +1740,13 @@
     </row>
     <row r="26" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>11</v>
@@ -1757,13 +1766,13 @@
     </row>
     <row r="27" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>11</v>
@@ -1783,13 +1792,13 @@
     </row>
     <row r="28" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>11</v>
@@ -1809,13 +1818,13 @@
     </row>
     <row r="29" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>11</v>
@@ -1835,13 +1844,13 @@
     </row>
     <row r="30" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>11</v>
@@ -1861,13 +1870,13 @@
     </row>
     <row r="31" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>11</v>
@@ -1887,13 +1896,13 @@
     </row>
     <row r="32" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>11</v>
@@ -1913,13 +1922,13 @@
     </row>
     <row r="33" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>11</v>
@@ -1939,13 +1948,13 @@
     </row>
     <row r="34" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>11</v>
@@ -1965,13 +1974,13 @@
     </row>
     <row r="35" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>11</v>
@@ -1991,13 +2000,13 @@
     </row>
     <row r="36" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>11</v>
@@ -2017,13 +2026,13 @@
     </row>
     <row r="37" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>11</v>
@@ -2043,13 +2052,13 @@
     </row>
     <row r="38" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>11</v>
@@ -2069,13 +2078,13 @@
     </row>
     <row r="39" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>11</v>
@@ -2095,13 +2104,13 @@
     </row>
     <row r="40" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>11</v>
@@ -2121,13 +2130,13 @@
     </row>
     <row r="41" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>11</v>
@@ -2147,13 +2156,13 @@
     </row>
     <row r="42" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>11</v>
@@ -2173,13 +2182,13 @@
     </row>
     <row r="43" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>11</v>
@@ -2199,13 +2208,13 @@
     </row>
     <row r="44" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>11</v>
@@ -2225,13 +2234,13 @@
     </row>
     <row r="45" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>11</v>
@@ -2251,13 +2260,13 @@
     </row>
     <row r="46" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>11</v>
@@ -2277,13 +2286,13 @@
     </row>
     <row r="47" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>11</v>
@@ -2303,13 +2312,13 @@
     </row>
     <row r="48" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>11</v>
@@ -2329,13 +2338,13 @@
     </row>
     <row r="49" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>11</v>
@@ -2355,13 +2364,13 @@
     </row>
     <row r="50" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>11</v>
@@ -2381,13 +2390,13 @@
     </row>
     <row r="51" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>11</v>
@@ -2407,13 +2416,13 @@
     </row>
     <row r="52" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>11</v>
@@ -2433,13 +2442,13 @@
     </row>
     <row r="53" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>11</v>
@@ -2459,13 +2468,13 @@
     </row>
     <row r="54" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>11</v>
@@ -2485,13 +2494,13 @@
     </row>
     <row r="55" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>11</v>
@@ -2511,13 +2520,13 @@
     </row>
     <row r="56" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>11</v>
@@ -2537,13 +2546,13 @@
     </row>
     <row r="57" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>11</v>
@@ -2563,13 +2572,13 @@
     </row>
     <row r="58" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>11</v>
@@ -2589,13 +2598,13 @@
     </row>
     <row r="59" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>11</v>
@@ -2615,13 +2624,13 @@
     </row>
     <row r="60" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>11</v>
@@ -2641,13 +2650,13 @@
     </row>
     <row r="61" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>11</v>
@@ -2667,13 +2676,13 @@
     </row>
     <row r="62" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>11</v>
@@ -2693,13 +2702,13 @@
     </row>
     <row r="63" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>11</v>
@@ -2719,13 +2728,13 @@
     </row>
     <row r="64" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>11</v>
@@ -2745,13 +2754,13 @@
     </row>
     <row r="65" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>11</v>
@@ -2771,13 +2780,13 @@
     </row>
     <row r="66" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>11</v>
@@ -2797,13 +2806,13 @@
     </row>
     <row r="67" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>11</v>
@@ -2823,13 +2832,13 @@
     </row>
     <row r="68" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>11</v>
@@ -2849,13 +2858,13 @@
     </row>
     <row r="69" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>11</v>
@@ -2875,13 +2884,13 @@
     </row>
     <row r="70" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>11</v>
@@ -2901,13 +2910,13 @@
     </row>
     <row r="71" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>11</v>
@@ -2927,13 +2936,13 @@
     </row>
     <row r="72" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D72" s="2" t="s">
         <v>11</v>
@@ -2953,13 +2962,13 @@
     </row>
     <row r="73" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>11</v>
@@ -2979,13 +2988,13 @@
     </row>
     <row r="74" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D74" s="2" t="s">
         <v>11</v>
@@ -3005,13 +3014,13 @@
     </row>
     <row r="75" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D75" s="2" t="s">
         <v>11</v>
@@ -3031,13 +3040,13 @@
     </row>
     <row r="76" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D76" s="2" t="s">
         <v>11</v>
@@ -3057,13 +3066,13 @@
     </row>
     <row r="77" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D77" s="2" t="s">
         <v>11</v>
@@ -3083,13 +3092,13 @@
     </row>
     <row r="78" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D78" s="2" t="s">
         <v>11</v>
@@ -3109,13 +3118,13 @@
     </row>
     <row r="79" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D79" s="2" t="s">
         <v>11</v>
@@ -3135,13 +3144,13 @@
     </row>
     <row r="80" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D80" s="2" t="s">
         <v>11</v>
@@ -3161,13 +3170,13 @@
     </row>
     <row r="81" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D81" s="2" t="s">
         <v>11</v>
@@ -3187,13 +3196,13 @@
     </row>
     <row r="82" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D82" s="2" t="s">
         <v>11</v>
@@ -3213,19 +3222,19 @@
     </row>
     <row r="83" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>10</v>
+        <v>112</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F83" s="2" t="s">
         <v>13</v>
@@ -3239,19 +3248,19 @@
     </row>
     <row r="84" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D84" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B84" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="C84" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D84" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="E84" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F84" s="2" t="s">
         <v>13</v>
@@ -3265,19 +3274,19 @@
     </row>
     <row r="85" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>10</v>
+        <v>112</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F85" s="2" t="s">
         <v>13</v>
@@ -3291,19 +3300,19 @@
     </row>
     <row r="86" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E86" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="B86" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="C86" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D86" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="E86" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="F86" s="2" t="s">
         <v>13</v>
@@ -3317,19 +3326,19 @@
     </row>
     <row r="87" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>10</v>
+        <v>112</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F87" s="2" t="s">
         <v>13</v>
@@ -3343,19 +3352,19 @@
     </row>
     <row r="88" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>10</v>
+        <v>112</v>
       </c>
       <c r="D88" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F88" s="2" t="s">
         <v>13</v>
@@ -3369,19 +3378,19 @@
     </row>
     <row r="89" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>10</v>
+        <v>112</v>
       </c>
       <c r="D89" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F89" s="2" t="s">
         <v>13</v>
@@ -3395,19 +3404,19 @@
     </row>
     <row r="90" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B90" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B90" s="2" t="s">
-        <v>120</v>
-      </c>
       <c r="C90" s="2" t="s">
-        <v>10</v>
+        <v>112</v>
       </c>
       <c r="D90" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F90" s="2" t="s">
         <v>13</v>
@@ -3421,19 +3430,19 @@
     </row>
     <row r="91" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>10</v>
+        <v>112</v>
       </c>
       <c r="D91" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F91" s="2" t="s">
         <v>13</v>
@@ -3447,13 +3456,13 @@
     </row>
     <row r="92" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>10</v>
+        <v>112</v>
       </c>
       <c r="D92" s="2" t="s">
         <v>11</v>
@@ -3462,7 +3471,7 @@
         <v>11</v>
       </c>
       <c r="F92" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G92" s="2" t="s">
         <v>11</v>
@@ -3473,13 +3482,13 @@
     </row>
     <row r="93" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B93" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="B93" s="2" t="s">
-        <v>125</v>
-      </c>
       <c r="C93" s="2" t="s">
-        <v>10</v>
+        <v>112</v>
       </c>
       <c r="D93" s="2" t="s">
         <v>11</v>
@@ -3488,7 +3497,7 @@
         <v>11</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G93" s="2" t="s">
         <v>11</v>
@@ -3499,22 +3508,22 @@
     </row>
     <row r="94" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F94" s="2" t="s">
         <v>128</v>
-      </c>
-      <c r="B94" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="C94" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D94" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E94" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F94" s="2" t="s">
-        <v>126</v>
       </c>
       <c r="G94" s="2" t="s">
         <v>11</v>
@@ -3525,13 +3534,13 @@
     </row>
     <row r="95" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>10</v>
+        <v>112</v>
       </c>
       <c r="D95" s="2" t="s">
         <v>11</v>
@@ -3540,7 +3549,7 @@
         <v>11</v>
       </c>
       <c r="F95" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G95" s="2" t="s">
         <v>11</v>
@@ -3551,22 +3560,22 @@
     </row>
     <row r="96" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>42</v>
+        <v>134</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="E96" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F96" s="2" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="G96" s="2" t="s">
         <v>11</v>
@@ -3577,22 +3586,22 @@
     </row>
     <row r="97" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C97" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="B97" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C97" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="D97" s="2" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="E97" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F97" s="2" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="G97" s="2" t="s">
         <v>11</v>
@@ -3603,22 +3612,22 @@
     </row>
     <row r="98" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D98" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="B98" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C98" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D98" s="2" t="s">
-        <v>132</v>
-      </c>
       <c r="E98" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F98" s="2" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="G98" s="2" t="s">
         <v>11</v>
@@ -3629,22 +3638,22 @@
     </row>
     <row r="99" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="E99" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F99" s="2" t="s">
         <v>136</v>
-      </c>
-      <c r="B99" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C99" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D99" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="E99" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F99" s="2" t="s">
-        <v>133</v>
       </c>
       <c r="G99" s="2" t="s">
         <v>11</v>
@@ -3655,13 +3664,13 @@
     </row>
     <row r="100" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D100" s="2" t="s">
         <v>11</v>
@@ -3681,13 +3690,13 @@
     </row>
     <row r="101" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="3" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D101" s="2" t="s">
         <v>11</v>
@@ -3707,13 +3716,13 @@
     </row>
     <row r="102" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="3" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D102" s="2" t="s">
         <v>11</v>
@@ -3733,13 +3742,13 @@
     </row>
     <row r="103" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D103" s="2" t="s">
         <v>11</v>
@@ -3759,13 +3768,13 @@
     </row>
     <row r="104" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="3" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D104" s="2" t="s">
         <v>11</v>
@@ -3785,13 +3794,13 @@
     </row>
     <row r="105" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="3" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D105" s="2" t="s">
         <v>11</v>
@@ -3811,13 +3820,13 @@
     </row>
     <row r="106" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="3" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D106" s="2" t="s">
         <v>11</v>
@@ -3837,13 +3846,13 @@
     </row>
     <row r="107" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="3" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D107" s="2" t="s">
         <v>11</v>
@@ -3863,13 +3872,13 @@
     </row>
     <row r="108" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="3" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D108" s="2" t="s">
         <v>11</v>
@@ -3889,13 +3898,13 @@
     </row>
     <row r="109" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="3" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D109" s="2" t="s">
         <v>11</v>
@@ -3915,13 +3924,13 @@
     </row>
     <row r="110" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="3" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D110" s="2" t="s">
         <v>11</v>
@@ -3941,13 +3950,13 @@
     </row>
     <row r="111" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="3" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D111" s="2" t="s">
         <v>11</v>
@@ -3967,13 +3976,13 @@
     </row>
     <row r="112" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="3" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D112" s="2" t="s">
         <v>11</v>
@@ -3993,13 +4002,13 @@
     </row>
     <row r="113" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="3" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D113" s="2" t="s">
         <v>11</v>
@@ -4019,13 +4028,13 @@
     </row>
     <row r="114" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="3" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D114" s="2" t="s">
         <v>11</v>
@@ -4045,13 +4054,13 @@
     </row>
     <row r="115" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="3" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D115" s="2" t="s">
         <v>11</v>
@@ -4071,13 +4080,13 @@
     </row>
     <row r="116" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="3" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D116" s="2" t="s">
         <v>11</v>
@@ -4097,13 +4106,13 @@
     </row>
     <row r="117" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="3" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D117" s="2" t="s">
         <v>11</v>
@@ -4123,13 +4132,13 @@
     </row>
     <row r="118" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="3" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D118" s="2" t="s">
         <v>11</v>
@@ -4149,13 +4158,13 @@
     </row>
     <row r="119" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="3" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D119" s="2" t="s">
         <v>11</v>
@@ -4175,13 +4184,13 @@
     </row>
     <row r="120" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="3" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D120" s="2" t="s">
         <v>11</v>
@@ -4201,13 +4210,13 @@
     </row>
     <row r="121" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="3" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D121" s="2" t="s">
         <v>11</v>
@@ -4227,13 +4236,13 @@
     </row>
     <row r="122" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="3" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D122" s="2" t="s">
         <v>11</v>
@@ -4253,13 +4262,13 @@
     </row>
     <row r="123" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="3" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D123" s="2" t="s">
         <v>11</v>
@@ -4279,13 +4288,13 @@
     </row>
     <row r="124" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="3" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D124" s="2" t="s">
         <v>11</v>
@@ -4305,13 +4314,13 @@
     </row>
     <row r="125" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="3" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D125" s="2" t="s">
         <v>11</v>
@@ -4331,13 +4340,13 @@
     </row>
     <row r="126" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="3" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D126" s="2" t="s">
         <v>11</v>
@@ -4357,13 +4366,13 @@
     </row>
     <row r="127" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="3" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D127" s="2" t="s">
         <v>11</v>
@@ -4383,13 +4392,13 @@
     </row>
     <row r="128" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="3" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D128" s="2" t="s">
         <v>11</v>
@@ -4409,13 +4418,13 @@
     </row>
     <row r="129" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="3" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D129" s="2" t="s">
         <v>11</v>
@@ -4435,13 +4444,13 @@
     </row>
     <row r="130" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="3" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D130" s="2" t="s">
         <v>11</v>
@@ -4461,13 +4470,13 @@
     </row>
     <row r="131" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="3" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D131" s="2" t="s">
         <v>11</v>
@@ -4487,13 +4496,13 @@
     </row>
     <row r="132" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="3" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D132" s="2" t="s">
         <v>11</v>
@@ -4513,13 +4522,13 @@
     </row>
     <row r="133" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="3" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D133" s="2" t="s">
         <v>11</v>
@@ -4539,13 +4548,13 @@
     </row>
     <row r="134" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="3" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D134" s="2" t="s">
         <v>11</v>
@@ -4565,13 +4574,13 @@
     </row>
     <row r="135" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="3" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D135" s="2" t="s">
         <v>11</v>
@@ -4591,13 +4600,13 @@
     </row>
     <row r="136" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="3" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D136" s="2" t="s">
         <v>11</v>
@@ -4617,13 +4626,13 @@
     </row>
     <row r="137" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="3" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D137" s="2" t="s">
         <v>11</v>
@@ -4643,13 +4652,13 @@
     </row>
     <row r="138" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="3" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D138" s="2" t="s">
         <v>11</v>
@@ -4669,13 +4678,13 @@
     </row>
     <row r="139" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A139" s="3" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D139" s="2" t="s">
         <v>11</v>
@@ -4695,13 +4704,13 @@
     </row>
     <row r="140" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A140" s="3" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D140" s="2" t="s">
         <v>11</v>
@@ -4721,13 +4730,13 @@
     </row>
     <row r="141" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A141" s="3" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D141" s="2" t="s">
         <v>11</v>
@@ -4747,13 +4756,13 @@
     </row>
     <row r="142" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A142" s="3" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D142" s="2" t="s">
         <v>11</v>
@@ -4773,13 +4782,13 @@
     </row>
     <row r="143" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A143" s="3" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D143" s="2" t="s">
         <v>11</v>
@@ -4799,13 +4808,13 @@
     </row>
     <row r="144" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A144" s="3" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D144" s="2" t="s">
         <v>11</v>
@@ -4825,13 +4834,13 @@
     </row>
     <row r="145" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A145" s="3" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D145" s="2" t="s">
         <v>11</v>
@@ -4851,13 +4860,13 @@
     </row>
     <row r="146" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A146" s="3" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D146" s="2" t="s">
         <v>11</v>
@@ -4877,13 +4886,13 @@
     </row>
     <row r="147" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A147" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D147" s="2" t="s">
         <v>11</v>
@@ -4903,13 +4912,13 @@
     </row>
     <row r="148" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A148" s="3" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D148" s="2" t="s">
         <v>11</v>
@@ -4929,13 +4938,13 @@
     </row>
     <row r="149" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A149" s="3" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D149" s="2" t="s">
         <v>11</v>
@@ -4955,13 +4964,13 @@
     </row>
     <row r="150" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A150" s="3" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D150" s="2" t="s">
         <v>11</v>
@@ -4981,13 +4990,13 @@
     </row>
     <row r="151" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A151" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D151" s="2" t="s">
         <v>11</v>
@@ -5007,13 +5016,13 @@
     </row>
     <row r="152" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A152" s="3" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D152" s="2" t="s">
         <v>11</v>
@@ -5033,13 +5042,13 @@
     </row>
     <row r="153" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A153" s="3" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D153" s="2" t="s">
         <v>11</v>
@@ -5059,13 +5068,13 @@
     </row>
     <row r="154" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A154" s="3" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D154" s="2" t="s">
         <v>11</v>
@@ -5085,13 +5094,13 @@
     </row>
     <row r="155" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A155" s="3" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D155" s="2" t="s">
         <v>11</v>
@@ -5111,13 +5120,13 @@
     </row>
     <row r="156" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A156" s="3" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D156" s="2" t="s">
         <v>11</v>
@@ -5137,13 +5146,13 @@
     </row>
     <row r="157" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A157" s="3" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D157" s="2" t="s">
         <v>11</v>
@@ -5163,13 +5172,13 @@
     </row>
     <row r="158" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A158" s="3" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D158" s="2" t="s">
         <v>11</v>
@@ -5189,13 +5198,13 @@
     </row>
     <row r="159" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A159" s="3" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D159" s="2" t="s">
         <v>11</v>
@@ -5215,13 +5224,13 @@
     </row>
     <row r="160" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A160" s="3" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D160" s="2" t="s">
         <v>11</v>
@@ -5241,13 +5250,13 @@
     </row>
     <row r="161" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A161" s="3" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D161" s="2" t="s">
         <v>11</v>
@@ -5267,13 +5276,13 @@
     </row>
     <row r="162" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A162" s="3" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D162" s="2" t="s">
         <v>11</v>
@@ -5293,13 +5302,13 @@
     </row>
     <row r="163" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A163" s="3" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D163" s="2" t="s">
         <v>11</v>
@@ -5319,13 +5328,13 @@
     </row>
     <row r="164" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A164" s="3" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D164" s="2" t="s">
         <v>11</v>
@@ -5345,22 +5354,22 @@
     </row>
     <row r="165" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A165" s="3" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>42</v>
+        <v>134</v>
       </c>
       <c r="D165" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E165" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="F165" s="2" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="G165" s="2" t="s">
         <v>11</v>
@@ -5371,22 +5380,22 @@
     </row>
     <row r="166" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A166" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="B166" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="B166" s="2" t="s">
-        <v>205</v>
-      </c>
       <c r="C166" s="2" t="s">
-        <v>42</v>
+        <v>134</v>
       </c>
       <c r="D166" s="2" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="E166" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="F166" s="2" t="s">
         <v>210</v>
-      </c>
-      <c r="F166" s="2" t="s">
-        <v>207</v>
       </c>
       <c r="G166" s="2" t="s">
         <v>11</v>
@@ -5397,22 +5406,22 @@
     </row>
     <row r="167" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A167" s="3" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>42</v>
+        <v>134</v>
       </c>
       <c r="D167" s="2" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="E167" s="2" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F167" s="2" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="G167" s="2" t="s">
         <v>11</v>
@@ -5423,22 +5432,22 @@
     </row>
     <row r="168" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A168" s="3" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>42</v>
+        <v>134</v>
       </c>
       <c r="D168" s="2" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="E168" s="2" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="F168" s="2" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="G168" s="2" t="s">
         <v>11</v>

</xml_diff>